<commit_message>
Lead machine: batch 1 bench matched by domain; tidy long owner titles
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VEQCtkhrjvn4vtJiWBdjLw
</commit_message>
<xml_diff>
--- a/lead-machine/batches/2026-10-12-E4L-Leads-batch1.xlsx
+++ b/lead-machine/batches/2026-10-12-E4L-Leads-batch1.xlsx
@@ -1094,7 +1094,7 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Attorney, Partner/Owner (About page: 'Meet Glen Howard, ESQ.' and experience list 'Howard Injury Law, Partner/Owner, Personal Injury Since 2017'); NV State Bar #9065, 'ATTORNEY Active', member since 10/20/2004, firm 'Law Offices of Glen A. Howard'; BBB lists 'Glen A. Howard, Attorney'</t>
+          <t>Attorney</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Owner / Member (founder per site schema 'Nikki Bridge'; registered agent of the LLC; BBB principal 'Nicole E. Bridge, Owner'). Co-owner: Kelly Bridge, 'HVAC Tech./Owner' (ROC record via BuildZoom; BBB 'Owner')</t>
+          <t>Owner / Member</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Owner/President (site 'Meet Our Staff' page: 'Mark Derringer Owner/President'; BBB Business Management: 'Mark Derringer, President'; quoted as 'Mark Derringer, President of Bob Heinmiller Air Conditioning' in the company's June 21, 2019 release). Co-owner: Linda Heinmiller(-Derringer), 'Owner/Corp. Secretary' on the site, 'Linda Derringer, Secretary' on BBB; she signs the About-Us letter and is the family-legacy voice. Founder: Bob Heinmiller.</t>
+          <t>Owner/President</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>President/Owner (BBB Business Management: 'Ryan Strache, President/Owner'); also Registered Agent of the GA corporation (OpenCorporates #0651574)</t>
+          <t>President/Owner</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Not found (no public page states a title; BBB lists 'Mr. Christian Shockley' as the contact with no title; Thumbtack profile 'Christian Shockley' uses first-person owner copy; GA SOS officers login-gated)</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Owner / Texas Master Electrician (site /residential-electrical-services: 'Todd Guernsey is a certified Master Electricians and owner of Light It Up Electric'; BBB 'Principal contacts: Todd Guernsey, Owner'; TDLR Master Electrician license ME 10479 'GUERNSEY, TODD D', Denton County, expires 04/08/2027; TX SOS registered agent 'Todd D Guernsey' for Light It Up Electric Inc.)</t>
+          <t>Owner / Texas Master Electrician</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Owner / Co-founder and Responsible Master Plumber (TSBPE license M-41669, Current). Site: "James and Dana Smith founded By The Book Plumbing".</t>
+          <t>Owner / Co-founder</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Owner (site About: "Matt Morgan — Owner"); "CEO/Owner" (BBB Business Management). Co-owners: Kristi Morgan (Owner) and Joey Wishnuck (Owner) — both on About page. CONFIRMED (site + BBB).</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Practice Owner and Veterinarian (site); President (BBB 'Business Management'); registered agent 'Johnson, Trish M' on the NC entity record (OpenCorporates us_nc/1154703)</t>
+          <t>Practice Owner</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>President/CFO (BBB); 'one of the owners' in her own words on the Aurora Chamber listing</t>
+          <t>President/CFO</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Owner (BBB 'Business Management: Cody Eason, Owner'; TN SOS registered agent at the LLC's head-office address per OpenCorporates; About-page photo caption 'Cody Eason - Hard at work'). Rutherford Chamber 'listed contact' NOT verifiable (page is JS-only). Second decision-maker: Jeremy Eason — 'Jeremy the owner was fantastic!' (Google review by 'Theo' on easonplumbing.com) and ProvenExpert contact person (no title). Cody PRIMARY (government + BBB), Jeremy LIKELY co-owner/family.</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Co-owner / co-founder (Marlin "Scott" Clark Sr.); co-owner Glenda Clark (bought her father's half in 2006, handles accounting); Marlin Clark Jr. 3rd generation (joined 2016) and registered agent of record</t>
+          <t>Co-owner / co-founder</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Owner (site: "assume ownership", Feb 2017) / President/CEO (BBB Business Management: "Casey M. Tynan")</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Orthodontist, DDS, MSD - leads the practice ("Led by... Dr. Fowler", "one-doctor, one-location practice"); registered agent of FOWLER ORTHODONTICS, PLLC as "CHAD E FOWLER" at the practice address. Explicit "owner" title not stated on site; OpenCorporates shows "1 officer" behind login.</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>President / Managing Member (BBB principal: "James A. Adams, President/Managing Member"); Master Electrician (site: "Master Electrician James Adams"; TDLR Master Electrician #220484, TECL #27762 on site); registered agent of ABR Electric LLC (OpenCorporates)</t>
+          <t>President / Managing Member</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Owner (BBB "Business Management": Abraham Valentin, Owner). Second decision-maker: Lelia Valentin, President (BBB) — corroborated as "LELIA M VALENTIN", registered agent of ABE'S ELECTRIC INC at 1004 Royal Street (Florida Sunbiz record via OpenCorporates). On-site Google reviews mention "Lisa and Abe" — recorded as-is, NOT reconciled with Lelia.</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Owner / Board Chair (site: "Dave Turner Owner/Board Chair", https://www.flobeds.com/about-us/); BBB lists "Mr. David R. Turner, President" (https://www.bbb.org/us/ca/fort-bragg/profile/mattress/flobeds-1116-15241). Day-to-day President is Dewey Turner (site), ~15 years in the family business.</t>
+          <t>Owner / Board Chair</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Founder / "matriarch" (About page; surname not published anywhere found). Family decision-makers also cited: Jana Marcelino — listed in BBB profile structured data as "Mrs. Jana Marcelino" (employee; no title shown) and LIKELY the daughter "Jana" named on About; Dannielli Marcelino, RN — master injector (LinkedIn company People tab + About "Dannielli RN"); Jeanie — Medical Consultant (About); Saharra — granddaughter, laser tech (About).</t>
+          <t>Founder / "matriarch"</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Owner / NC Heating Contractor license holder (Groups 1, 2, 3) — LinkedIn headline 'Small Business Owner'; Yelp 'Business Owner'; NC Board record lists 'Contact Name: Robert Allen George' for AirPro Carolina, LLC; OpenCorporates registered agent 'George, Robert Allen'; Google Ads verified advertiser legal name 'Robert A George'</t>
+          <t>Owner / NC Heating Contractor license holder</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Owner / Member (BBB Business Management) and AZ ROC Qualifying Party (BuildZoom); customers call him 'the owner Josh'; Apr-2024 press release calls him 'founder and CEO'</t>
+          <t>Owner / Member</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Owner / President ("Hey guys, this is Ricky, owner of AirBros Air Conditioning and Electrical" on the site; BBB lists "Ricardo Orta, President"; OpenCorporates registered agent "RICARDO A ORTA")</t>
+          <t>Owner / President</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Founder (About page: 'Howard Manne established The Electrician in 2004'; 'family-owned and operated'). No formal title published - 'Owner' is inferred, not stated.</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Owner / Master Plumber (BBB: "Trent Cooke, Owner"; site About: "co-owners, Charles Wallace and Trent Cooke"; SOS via OpenCorporates: registered agent "Trent A Cooke"; 2022 press release: "owner Trent Cooke"). Co-owner: Charles Wallace (site About; LinkedIn company page).</t>
+          <t>Owner / Master Plumber</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>President (BBB principal contact: 'Bill West, President' — https://www.bbb.org/us/mo/grain-valley/profile/roofing-contractors/bill-west-roofing-inc-0714-97101169); Founder/owner per site ('Founded by Bill West and now operated alongside his son Aaron' — home; 'Today Bill and his son Aaron oversee Bill West Roofing, Inc.' — /about-us/). Second decision-maker: Aaron (son; runs estimates and customer education per /about-us/; surname NOT published on any page found — do not assume).</t>
+          <t>President</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>Attorney, Partner/Owner (About page: 'Meet Glen Howard, ESQ.' and experience list 'Howard Injury Law, Partner/Owner, Personal Injury Since 2017'); NV State Bar #9065, 'ATTORNEY Active', member since 10/20/2004, firm 'Law Offices of Glen A. Howard'; BBB lists 'Glen A. Howard, Attorney'</t>
+          <t>Attorney</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="BQ2" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: NV Bar firm name: Law Offices of Glen A. Howard. Band: QUALIFIED (71, TRUSTED) - not SEND TODAY only because the D4 AI spot-check could not be run this session; run the 28-answer GEO audit and build the bilingual voice demo before first touch, then re-band. Route: email-first to ghoward@ (Confirmed personal email, Google Workspace MX) with Sam's call within 48h, Tue-Thu 9-10:30 AM PT. Compliance: legal vertical - no outcomes, no legal advice, no case-volume promises; never quote the 'personal cell' review back to him or name reviewers. Watch-outs: (1) Storm Media (his agency) advertises 'SEO + GEO + AEO' and the site already has FAQ/LegalService/Attorney schema - expect the GEO audit to show partial presence; the phone gap is the cleaner wedge. (2) Intaker sells an 'AI Texting Agent' - confirm on the call whether he uses it before pitching missed-call text-back as new. (3) Demo must handle Spanish at minimum (site also promises Cantonese and Mandarin). (4) Vanessa Kitchen (ex-practice administrator with marketing background) is the likely internal champion. Not verifiable this session (blocked/403/JS): Google review replies and lowest-rated reviews, Yelp, Avvo, Indeed/job posts, Meta Ad Library, Google Ads Transparency, LSA badge, LinkedIn, Nevada SOS, Facebook/Instagram/TikTok recency - refresh D3/D6 if a slot depends on them.</t>
+          <t>Title detail: Attorney, Partner/Owner (About page: 'Meet Glen Howard, ESQ.' and experience list 'Howard Injury Law, Partner/Owner, Personal Injury Since 2017'); NV State Bar #9065, 'ATTORNEY Active', member since 10/20/2004, firm 'Law Offices of Glen A. Howard'; BBB lists 'Glen A. Howard, Attorney'. Legal entity note: NV Bar firm name: Law Offices of Glen A. Howard. Band: QUALIFIED (71, TRUSTED) - not SEND TODAY only because the D4 AI spot-check could not be run this session; run the 28-answer GEO audit and build the bilingual voice demo before first touch, then re-band. Route: email-first to ghoward@ (Confirmed personal email, Google Workspace MX) with Sam's call within 48h, Tue-Thu 9-10:30 AM PT. Compliance: legal vertical - no outcomes, no legal advice, no case-volume promises; never quote the 'personal cell' review back to him or name reviewers. Watch-outs: (1) Storm Media (his agency) advertises 'SEO + GEO + AEO' and the site already has FAQ/LegalService/Attorney schema - expect the GEO audit to show partial presence; the phone gap is the cleaner wedge. (2) Intaker sells an 'AI Texting Agent' - confirm on the call whether he uses it before pitching missed-call text-back as new. (3) Demo must handle Spanish at minimum (site also promises Cantonese and Mandarin). (4) Vanessa Kitchen (ex-practice administrator with marketing background) is the likely internal champion. Not verifiable this session (blocked/403/JS): Google review replies and lowest-rated reviews, Yelp, Avvo, Indeed/job posts, Meta Ad Library, Google Ads Transparency, LSA badge, LinkedIn, Nevada SOS, Facebook/Instagram/TikTok recency - refresh D3/D6 if a slot depends on them.</t>
         </is>
       </c>
       <c r="BR2" s="10" t="inlineStr"/>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>Owner / Member (founder per site schema 'Nikki Bridge'; registered agent of the LLC; BBB principal 'Nicole E. Bridge, Owner'). Co-owner: Kelly Bridge, 'HVAC Tech./Owner' (ROC record via BuildZoom; BBB 'Owner')</t>
+          <t>Owner / Member</t>
         </is>
       </c>
       <c r="L3" s="8" t="inlineStr">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="BQ3" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: Viking Heating and Air Conditioning, LLC. Second decision-maker: Kelly Bridge, 'HVAC Tech./Owner' (likely in the field) - Nicole/Nikki is the registered agent and schema founder, so she is the better first ask; license qualifying party is Joel Montoya (not an owner). Email is generic info@ only - route to Sam first; if emailing, write for a gatekeeper and ask for Nikki or Kelly. Best call window (AZ, no DST, MST): trades 7:00-8:30am or 4:00-5:30pm. Phone 480-689-5167 is consistent across site, BBB and BuildZoom (CallRail present, but this appears to be the main line, not a swapped tracking number). Marketing stack signals an unnamed vendor (CallRail, Meta pixel, automated weather-triggered blog at blog.viking-hvac.com, 8 LinkedIn posts in 10 days) - ask 'who runs your blog and ads?' before pitching GEO; FAQPage schema already on the homepage. Watch-outs: review reply tone unknown (could not render Google replies); 'Best of business rate 2024/2025' badge issuer not identified; the Oct 2025 commercial-expansion PR now 404s (do not cite it as current); a technician named Logan Bridge appears in an Oct 2, 2026 review - do not assume any relation. Before loading to GHL: run ghl-contacts.js dedupe (domain viking-hvac.com / 480-689-5167 / name+Chandler); run the D4 AI spot-check (3 money questions x 2 platforms) to see if this can move to SEND TODAY. Compliance: no cell numbers found; main line is a business line; no 'no solicitation' notice seen.</t>
+          <t>Title detail: Owner / Member (founder per site schema 'Nikki Bridge'; registered agent of the LLC; BBB principal 'Nicole E. Bridge, Owner'). Co-owner: Kelly Bridge, 'HVAC Tech./Owner' (ROC record via BuildZoom; BBB 'Owner'). Legal entity note: legal: Viking Heating and Air Conditioning, LLC. Second decision-maker: Kelly Bridge, 'HVAC Tech./Owner' (likely in the field) - Nicole/Nikki is the registered agent and schema founder, so she is the better first ask; license qualifying party is Joel Montoya (not an owner). Email is generic info@ only - route to Sam first; if emailing, write for a gatekeeper and ask for Nikki or Kelly. Best call window (AZ, no DST, MST): trades 7:00-8:30am or 4:00-5:30pm. Phone 480-689-5167 is consistent across site, BBB and BuildZoom (CallRail present, but this appears to be the main line, not a swapped tracking number). Marketing stack signals an unnamed vendor (CallRail, Meta pixel, automated weather-triggered blog at blog.viking-hvac.com, 8 LinkedIn posts in 10 days) - ask 'who runs your blog and ads?' before pitching GEO; FAQPage schema already on the homepage. Watch-outs: review reply tone unknown (could not render Google replies); 'Best of business rate 2024/2025' badge issuer not identified; the Oct 2025 commercial-expansion PR now 404s (do not cite it as current); a technician named Logan Bridge appears in an Oct 2, 2026 review - do not assume any relation. Before loading to GHL: run ghl-contacts.js dedupe (domain viking-hvac.com / 480-689-5167 / name+Chandler); run the D4 AI spot-check (3 money questions x 2 platforms) to see if this can move to SEND TODAY. Compliance: no cell numbers found; main line is a business line; no 'no solicitation' notice seen.</t>
         </is>
       </c>
       <c r="BR3" s="10" t="inlineStr"/>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>Owner/President (site 'Meet Our Staff' page: 'Mark Derringer Owner/President'; BBB Business Management: 'Mark Derringer, President'; quoted as 'Mark Derringer, President of Bob Heinmiller Air Conditioning' in the company's June 21, 2019 release). Co-owner: Linda Heinmiller(-Derringer), 'Owner/Corp. Secretary' on the site, 'Linda Derringer, Secretary' on BBB; she signs the About-Us letter and is the family-legacy voice. Founder: Bob Heinmiller.</t>
+          <t>Owner/President</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="BQ4" s="8" t="inlineStr">
         <is>
-          <t>1) Address Mark Derringer as Owner/President; Linda Heinmiller(-Derringer), Owner/Corp. Secretary, signs the family letter - consider copying her on email; do not characterize their relationship beyond 'co-owners'. 2) Only a generic mailbox exists (service@) - route call-first; if emailing, write for a gatekeeper and ask for Mark by name. 3) Never quote the 'will not call me back' or 'call me back this afternoon' reviews verbatim to the owner; summarize as a pattern. 4) Do not imply replacing office staff - position as after-hours/overflow only (Family-Legacy playbook). 5) Not verified from here: GBP hours and owner-reply rate (Google blocked), Google Ads / Meta Ad Library / LSA (blocked), ChatGPT/Perplexity/Gemini spot-check (blocked - only one platform checked). 6) A directory shows license CAC057411 'exp 08/31/2026'; DBPR search returned no record for my query - verify renewal on myfloridalicense.com before citing the license. 7) Sister entity Bob Heinmiller Solar Solutions, LLC (1519 W Smith St, Birdeye-managed reviews, Mon-Fri 8-5) shares the owners - one demo line could cover AC + electrical + solar intake. 8) Carrier's dealer page shows a different phone (321-319-3980) - they may already have a dealer-locator tracking line; ask, don't assume. 9) Suppression.csv and seen.csv are clean; GHL E4L Services dedupe (ghl-contacts.js) still needs to run before load. 10) Florida call window is 8 AM-8 PM; Sam should log who answers (human/IVR/voicemail) to update D2.</t>
+          <t>Title detail: Owner/President (site 'Meet Our Staff' page: 'Mark Derringer Owner/President'; BBB Business Management: 'Mark Derringer, President'; quoted as 'Mark Derringer, President of Bob Heinmiller Air Conditioning' in the company's June 21, 2019 release). Co-owner: Linda Heinmiller(-Derringer), 'Owner/Corp. Secretary' on the site, 'Linda Derringer, Secretary' on BBB; she signs the About-Us letter and is the family-legacy voice. Founder: Bob Heinmiller.. 1) Address Mark Derringer as Owner/President; Linda Heinmiller(-Derringer), Owner/Corp. Secretary, signs the family letter - consider copying her on email; do not characterize their relationship beyond 'co-owners'. 2) Only a generic mailbox exists (service@) - route call-first; if emailing, write for a gatekeeper and ask for Mark by name. 3) Never quote the 'will not call me back' or 'call me back this afternoon' reviews verbatim to the owner; summarize as a pattern. 4) Do not imply replacing office staff - position as after-hours/overflow only (Family-Legacy playbook). 5) Not verified from here: GBP hours and owner-reply rate (Google blocked), Google Ads / Meta Ad Library / LSA (blocked), ChatGPT/Perplexity/Gemini spot-check (blocked - only one platform checked). 6) A directory shows license CAC057411 'exp 08/31/2026'; DBPR search returned no record for my query - verify renewal on myfloridalicense.com before citing the license. 7) Sister entity Bob Heinmiller Solar Solutions, LLC (1519 W Smith St, Birdeye-managed reviews, Mon-Fri 8-5) shares the owners - one demo line could cover AC + electrical + solar intake. 8) Carrier's dealer page shows a different phone (321-319-3980) - they may already have a dealer-locator tracking line; ask, don't assume. 9) Suppression.csv and seen.csv are clean; GHL E4L Services dedupe (ghl-contacts.js) still needs to run before load. 10) Florida call window is 8 AM-8 PM; Sam should log who answers (human/IVR/voicemail) to update D2.</t>
         </is>
       </c>
       <c r="BR4" s="10" t="inlineStr"/>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>President/Owner (BBB Business Management: 'Ryan Strache, President/Owner'); also Registered Agent of the GA corporation (OpenCorporates #0651574)</t>
+          <t>President/Owner</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="BQ5" s="8" t="inlineStr">
         <is>
-          <t>1) Band = QUALIFIED (70, TRUSTED on 6/7 dimensions) but held out of SEND TODAY only because the D4 AI spot-check could not run this turn (web-search budget exhausted; AI platforms not reachable) — one Perplexity/ChatGPT pass on 'emergency tree removal near Kennesaw, GA' promotes it. 2) GHL 'E4L Services' dedupe (ghl-contacts.js by domain/phone/name+city) was NOT run from this subagent; suppression.csv and seen.csv are clean (0 hits for name, domain, Strache). 3) Email route: ryan@appalachiantreeservice.com is Confirmed (on the business's own site + JSON-LD, Google Workspace MX); send from Sebastian plain-text, Sam calls within 48 h. 4) Google/Yelp/Angi/HomeAdvisor reviews and Facebook/Instagram/X could not be opened (403/login walls), so review-reply behavior and social cadence are unknown — Rozel may want a quick manual look at the GBP before send. 5) The site is built on Manus (AI website builder) — he has already used an AI tool, so 'AI' is not a scary word, but lead with the 9 PM storm call, not the tech. 6) Do not say he misses calls (Nextdoor praises his response speed); frame as after-hours and storm-surge coverage. 7) OpenCorporates lists the registered agent at a non-business address — not recorded, do not use. 8) Demo scenario for Abdullah: tree on the house after a storm at night; AI collects name, number, address, what fell, offers the free estimate and books the next-morning assessment; no nighttime dispatch promised. 9) Referral partners on his site (roofing, HVAC, landscaping, stump grinding, arborist) are a possible referral angle later — the HVAC partner (Top Tech Mechanical) advertises 24-hour emergency service, a natural contrast he will recognize.</t>
+          <t>Title detail: President/Owner (BBB Business Management: 'Ryan Strache, President/Owner'); also Registered Agent of the GA corporation (OpenCorporates #0651574). 1) Band = QUALIFIED (70, TRUSTED on 6/7 dimensions) but held out of SEND TODAY only because the D4 AI spot-check could not run this turn (web-search budget exhausted; AI platforms not reachable) — one Perplexity/ChatGPT pass on 'emergency tree removal near Kennesaw, GA' promotes it. 2) GHL 'E4L Services' dedupe (ghl-contacts.js by domain/phone/name+city) was NOT run from this subagent; suppression.csv and seen.csv are clean (0 hits for name, domain, Strache). 3) Email route: ryan@appalachiantreeservice.com is Confirmed (on the business's own site + JSON-LD, Google Workspace MX); send from Sebastian plain-text, Sam calls within 48 h. 4) Google/Yelp/Angi/HomeAdvisor reviews and Facebook/Instagram/X could not be opened (403/login walls), so review-reply behavior and social cadence are unknown — Rozel may want a quick manual look at the GBP before send. 5) The site is built on Manus (AI website builder) — he has already used an AI tool, so 'AI' is not a scary word, but lead with the 9 PM storm call, not the tech. 6) Do not say he misses calls (Nextdoor praises his response speed); frame as after-hours and storm-surge coverage. 7) OpenCorporates lists the registered agent at a non-business address — not recorded, do not use. 8) Demo scenario for Abdullah: tree on the house after a storm at night; AI collects name, number, address, what fell, offers the free estimate and books the next-morning assessment; no nighttime dispatch promised. 9) Referral partners on his site (roofing, HVAC, landscaping, stump grinding, arborist) are a possible referral angle later — the HVAC partner (Top Tech Mechanical) advertises 24-hour emergency service, a natural contrast he will recognize.</t>
         </is>
       </c>
       <c r="BR5" s="10" t="inlineStr"/>
@@ -6606,7 +6606,7 @@
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Not found (no public page states a title; BBB lists 'Mr. Christian Shockley' as the contact with no title; Thumbtack profile 'Christian Shockley' uses first-person owner copy; GA SOS officers login-gated)</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="L7" s="8" t="inlineStr">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="BQ7" s="8" t="inlineStr">
         <is>
-          <t>(1) GHL 'E4L Services' dedupe (ghl-contacts.js by domain/phone/name+city) was NOT run in this session — run before load. (2) Title is not formally cited anywhere; GA SOS officer names are login-gated on OpenCorporates and ecorp.sos.ga.gov served a JS challenge. Address him as 'Christian' (email handle, Thumbtack name, reviews); his legal first name may be Jon (WP author 'Jon Shockley', review 'Christian (Jon)'). Don't write 'Owner' in copy until SOS confirms. (3) License EN216228 is self-published; GA license board lookup not checked. (4) Possible second person: a Nextdoor user from Hiram, GA posts in first person for the business ('Give us a call! Shockley Electric, it's something we do all the time') — initials only, unverified; Sam should ask 'who else helps with the phones?' (5) Web vendor: the site's public author list shows a 'Green Mellen' account (GreenMellen Media, Marietta) — don't lead with a site rebuild; GEO/schema is the wedge there. (6) Google review count conflicts (90 / 180 / 477) — verify on Maps before quoting. (7) Home-based: BBB, Nextdoor and SOS addresses all differ — never reference an address. (8) Best call window: 7:00–8:30 AM or 4:00–5:30 PM ET, Mon–Fri (hours 9–5:30). Main line may be his cell — manual dial only, no SMS/AI outbound. (9) Demo build notes: include EV charger and generator inquiries even though the site doesn't list them (ask on the call if he does them), route 'sparking/burning smell' to urgent, capture panel-upgrade estimate requests, mention the lifetime labor guarantee in the greeting. (10) Tone: terse, anti-upsell ('we do not upsell', 'we will never oversell you') — keep the email under 90 words, no hype, no 'AI' in the subject. (11) Facebook, Google reviews, LinkedIn, Meta Ad Library, Ads Transparency, LSA and the AI spot-check were all inaccessible this session; re-run D4 before SEND TODAY promotion.</t>
+          <t>Title detail: Not found (no public page states a title; BBB lists 'Mr. Christian Shockley' as the contact with no title; Thumbtack profile 'Christian Shockley' uses first-person owner copy; GA SOS officers login-gated). (1) GHL 'E4L Services' dedupe (ghl-contacts.js by domain/phone/name+city) was NOT run in this session — run before load. (2) Title is not formally cited anywhere; GA SOS officer names are login-gated on OpenCorporates and ecorp.sos.ga.gov served a JS challenge. Address him as 'Christian' (email handle, Thumbtack name, reviews); his legal first name may be Jon (WP author 'Jon Shockley', review 'Christian (Jon)'). Don't write 'Owner' in copy until SOS confirms. (3) License EN216228 is self-published; GA license board lookup not checked. (4) Possible second person: a Nextdoor user from Hiram, GA posts in first person for the business ('Give us a call! Shockley Electric, it's something we do all the time') — initials only, unverified; Sam should ask 'who else helps with the phones?' (5) Web vendor: the site's public author list shows a 'Green Mellen' account (GreenMellen Media, Marietta) — don't lead with a site rebuild; GEO/schema is the wedge there. (6) Google review count conflicts (90 / 180 / 477) — verify on Maps before quoting. (7) Home-based: BBB, Nextdoor and SOS addresses all differ — never reference an address. (8) Best call window: 7:00–8:30 AM or 4:00–5:30 PM ET, Mon–Fri (hours 9–5:30). Main line may be his cell — manual dial only, no SMS/AI outbound. (9) Demo build notes: include EV charger and generator inquiries even though the site doesn't list them (ask on the call if he does them), route 'sparking/burning smell' to urgent, capture panel-upgrade estimate requests, mention the lifetime labor guarantee in the greeting. (10) Tone: terse, anti-upsell ('we do not upsell', 'we will never oversell you') — keep the email under 90 words, no hype, no 'AI' in the subject. (11) Facebook, Google reviews, LinkedIn, Meta Ad Library, Ads Transparency, LSA and the AI spot-check were all inaccessible this session; re-run D4 before SEND TODAY promotion.</t>
         </is>
       </c>
       <c r="BR7" s="10" t="inlineStr"/>
@@ -6947,7 +6947,7 @@
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>Owner / Texas Master Electrician (site /residential-electrical-services: 'Todd Guernsey is a certified Master Electricians and owner of Light It Up Electric'; BBB 'Principal contacts: Todd Guernsey, Owner'; TDLR Master Electrician license ME 10479 'GUERNSEY, TODD D', Denton County, expires 04/08/2027; TX SOS registered agent 'Todd D Guernsey' for Light It Up Electric Inc.)</t>
+          <t>Owner / Texas Master Electrician</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
@@ -7237,7 +7237,7 @@
       </c>
       <c r="BQ8" s="8" t="inlineStr">
         <is>
-          <t>1) Route: QUALIFIED (66, TRUSTED). D1 = 14 via LinkedIn + generic mailbox, so the email goes to Info@ (gatekeeper-friendly copy) with a same-week Sam call; demo_build = yes (phone-first, site scrapable). 2) D4 was NOT run — no AI platform was reachable this session; a GEO spot-check for 'EV charger installer Frisco, TX' could add up to 6 points and gives ask #2. 3) Review-reply behavior, Facebook/LinkedIn content, hiring, and ad activity are all unverified (Google Maps JS shell, Yelp/Angi/Indeed 403, Facebook login wall, LinkedIn 999, Meta Ad Library 403, Ads Transparency JS-only, Wayback unavailable); the Google Ads conversion tag is the only spend proof. 4) Conflicts to be aware of: founded 'since 2000' vs TX corp trading-name date 2005-04-26 vs domain 2006 (likely sole prop → Inc.); review count 252 (site schema) vs Google 74 (expertise.com); reception hours 8–5 (contact page) vs 9–5 (appointment page). 5) Natasha Guernsey writes the blog twice a week in a warm, emoji-heavy voice — she is the content/marketing voice and a plausible champion; Todd is the technical owner (master license holder). Do not reference family ties. 6) Niche read: technical and allergic to hype — lead with the demo number and the after-5 gap, keep 'AI' out of the subject line, no feature lists. 7) Natural tie-in: the receptionist can offer the Advantage Plan ($179/yr) to after-hours callers — frame as protecting the membership push they are already making. 8) The 'Voted Best Electrician in Frisco' award is undated and the awarding body was not found; use it softly or not at all.</t>
+          <t>Title detail: Owner / Texas Master Electrician (site /residential-electrical-services: 'Todd Guernsey is a certified Master Electricians and owner of Light It Up Electric'; BBB 'Principal contacts: Todd Guernsey, Owner'; TDLR Master Electrician license ME 10479 'GUERNSEY, TODD D', Denton County, expires 04/08/2027; TX SOS registered agent 'Todd D Guernsey' for Light It Up Electric Inc.). 1) Route: QUALIFIED (66, TRUSTED). D1 = 14 via LinkedIn + generic mailbox, so the email goes to Info@ (gatekeeper-friendly copy) with a same-week Sam call; demo_build = yes (phone-first, site scrapable). 2) D4 was NOT run — no AI platform was reachable this session; a GEO spot-check for 'EV charger installer Frisco, TX' could add up to 6 points and gives ask #2. 3) Review-reply behavior, Facebook/LinkedIn content, hiring, and ad activity are all unverified (Google Maps JS shell, Yelp/Angi/Indeed 403, Facebook login wall, LinkedIn 999, Meta Ad Library 403, Ads Transparency JS-only, Wayback unavailable); the Google Ads conversion tag is the only spend proof. 4) Conflicts to be aware of: founded 'since 2000' vs TX corp trading-name date 2005-04-26 vs domain 2006 (likely sole prop → Inc.); review count 252 (site schema) vs Google 74 (expertise.com); reception hours 8–5 (contact page) vs 9–5 (appointment page). 5) Natasha Guernsey writes the blog twice a week in a warm, emoji-heavy voice — she is the content/marketing voice and a plausible champion; Todd is the technical owner (master license holder). Do not reference family ties. 6) Niche read: technical and allergic to hype — lead with the demo number and the after-5 gap, keep 'AI' out of the subject line, no feature lists. 7) Natural tie-in: the receptionist can offer the Advantage Plan ($179/yr) to after-hours callers — frame as protecting the membership push they are already making. 8) The 'Voted Best Electrician in Frisco' award is undated and the awarding body was not found; use it softly or not at all.</t>
         </is>
       </c>
       <c r="BR8" s="10" t="inlineStr"/>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
-          <t>Owner / Co-founder and Responsible Master Plumber (TSBPE license M-41669, Current). Site: "James and Dana Smith founded By The Book Plumbing".</t>
+          <t>Owner / Co-founder</t>
         </is>
       </c>
       <c r="L9" s="8" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="BQ9" s="8" t="inlineStr">
         <is>
-          <t>Second decision-maker: Dana Smith, co-founder per the About page ("James and Dana Smith"); relationship beyond "family-run" is not stated, so address James and mention Dana only if she picks up. Best call window (Central): 7:00-8:30am or 4:00-5:30pm (GBP hours end at 4pm; he likely answers his own line). Main line 281-907-2092 is the only published number and may be the owner's own phone - manual human dial only, no SMS or AI voice. Entity: By The Book Plumbing LLC, TX file no. 0802827696, status "In Existence", registered agent James A Smith, 6311 Cobble Manor Ln, Spring TX 77379 (OpenCorporates mirror; officer list login-gated; PIRs filed through 2024). License: TSBPE Responsible Master Plumber M-41669, SMITH JAMES ALLEN, Current, issued 07/18/2016, expires 10/31/2026, insurer State Farm (RMP list dated 2026-10-08) - renewal window is open now, a natural "tidying the business" moment. Not a franchise, no chain hints, one location. BBB: no profile. Approach: do not open with "AI"; open with the Saturday/after-4pm call and the demo number; neighbors call him "old school" and he is code-driven, so stress the agent is trained on his site and answers as By The Book. Do not imply his reviews show a problem - they do not; frame as capacity and overflow. Price sensitivity: 5% cash/check discount and Wisetack financing suggest margin-aware; frame Recover around one recovered water-heater job per month, no numbers promised. The "$600 Federal Tax Credit on Tankless Water Heaters" banner is a safe alternate opener, but do not make tax claims ourselves. Gaps to close before send: (1) GEO audit (D4 unchecked - web search budget exhausted); (2) GHL E4L Services dedupe via ghl-contacts.js; (3) Facebook page is login-walled - check for recent owner posts by hand; (4) Yelp, LinkedIn X-ray, Indeed, LSA, and ad libraries could not be checked this run; (5) Bradford White dealer page from the scout (Magnolia TX address) returned 403 and is unverified. Compliance: no sensitive data recorded; registered address appears residential, do not use for mail or visits.</t>
+          <t>Title detail: Owner / Co-founder and Responsible Master Plumber (TSBPE license M-41669, Current). Site: "James and Dana Smith founded By The Book Plumbing".. Second decision-maker: Dana Smith, co-founder per the About page ("James and Dana Smith"); relationship beyond "family-run" is not stated, so address James and mention Dana only if she picks up. Best call window (Central): 7:00-8:30am or 4:00-5:30pm (GBP hours end at 4pm; he likely answers his own line). Main line 281-907-2092 is the only published number and may be the owner's own phone - manual human dial only, no SMS or AI voice. Entity: By The Book Plumbing LLC, TX file no. 0802827696, status "In Existence", registered agent James A Smith, 6311 Cobble Manor Ln, Spring TX 77379 (OpenCorporates mirror; officer list login-gated; PIRs filed through 2024). License: TSBPE Responsible Master Plumber M-41669, SMITH JAMES ALLEN, Current, issued 07/18/2016, expires 10/31/2026, insurer State Farm (RMP list dated 2026-10-08) - renewal window is open now, a natural "tidying the business" moment. Not a franchise, no chain hints, one location. BBB: no profile. Approach: do not open with "AI"; open with the Saturday/after-4pm call and the demo number; neighbors call him "old school" and he is code-driven, so stress the agent is trained on his site and answers as By The Book. Do not imply his reviews show a problem - they do not; frame as capacity and overflow. Price sensitivity: 5% cash/check discount and Wisetack financing suggest margin-aware; frame Recover around one recovered water-heater job per month, no numbers promised. The "$600 Federal Tax Credit on Tankless Water Heaters" banner is a safe alternate opener, but do not make tax claims ourselves. Gaps to close before send: (1) GEO audit (D4 unchecked - web search budget exhausted); (2) GHL E4L Services dedupe via ghl-contacts.js; (3) Facebook page is login-walled - check for recent owner posts by hand; (4) Yelp, LinkedIn X-ray, Indeed, LSA, and ad libraries could not be checked this run; (5) Bradford White dealer page from the scout (Magnolia TX address) returned 403 and is unverified. Compliance: no sensitive data recorded; registered address appears residential, do not use for mail or visits.</t>
         </is>
       </c>
       <c r="BR9" s="10" t="inlineStr"/>
@@ -7629,7 +7629,7 @@
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>Owner (site About: "Matt Morgan — Owner"); "CEO/Owner" (BBB Business Management). Co-owners: Kristi Morgan (Owner) and Joey Wishnuck (Owner) — both on About page. CONFIRMED (site + BBB).</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
@@ -7919,7 +7919,7 @@
       </c>
       <c r="BQ10" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: ScissorTail Roofing and Construction LLC per BBB. (1) Three owners: Matt Morgan is founder/CEO and media contact; Kristi Morgan (co-owner) has the marketing background per About — she may own the marketing-spend decision, so address Matt and copy/ask for Kristi on the Game Plan Call; Joey Wishnuck is an investor/developer with other ventures. (2) The only published email is Matt Seaton's (Director of Operations) — route the demo link through him as champion; do not address him as owner. (3) Do not open with reviews — none were readable this run; verify GBP (4.9/99 is site-claimed) before quoting anything. (4) GEO is NOT the opener: site already carries FAQPage/LocalBusiness schema and allowlists GPTBot/ClaudeBot; run the D4 spot-check before any "Named in X of Y" line. (5) Oklahoma has telemarketer-registration/mini-TCPA rules — confirm compliance before Sam dials (playbook legal section). (6) (405) 452-0591 is unverified line type — manual human dial only, no SMS. (7) GHL 'E4L Services' dedupe was not run by this agent (no access) — run ghl-contacts.js by domain/phone/name+city before loading. (8) Avoid any mention of the site's /review/ page sentiment-gating. (9) About page contains family/church details — excluded here; do not use in outreach.</t>
+          <t>Title detail: Owner (site About: "Matt Morgan — Owner"); "CEO/Owner" (BBB Business Management). Co-owners: Kristi Morgan (Owner) and Joey Wishnuck (Owner) — both on About page. CONFIRMED (site + BBB).. Legal entity note: legal: ScissorTail Roofing and Construction LLC per BBB. (1) Three owners: Matt Morgan is founder/CEO and media contact; Kristi Morgan (co-owner) has the marketing background per About — she may own the marketing-spend decision, so address Matt and copy/ask for Kristi on the Game Plan Call; Joey Wishnuck is an investor/developer with other ventures. (2) The only published email is Matt Seaton's (Director of Operations) — route the demo link through him as champion; do not address him as owner. (3) Do not open with reviews — none were readable this run; verify GBP (4.9/99 is site-claimed) before quoting anything. (4) GEO is NOT the opener: site already carries FAQPage/LocalBusiness schema and allowlists GPTBot/ClaudeBot; run the D4 spot-check before any "Named in X of Y" line. (5) Oklahoma has telemarketer-registration/mini-TCPA rules — confirm compliance before Sam dials (playbook legal section). (6) (405) 452-0591 is unverified line type — manual human dial only, no SMS. (7) GHL 'E4L Services' dedupe was not run by this agent (no access) — run ghl-contacts.js by domain/phone/name+city before loading. (8) Avoid any mention of the site's /review/ page sentiment-gating. (9) About page contains family/church details — excluded here; do not use in outreach.</t>
         </is>
       </c>
       <c r="BR10" s="10" t="inlineStr"/>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>Practice Owner and Veterinarian (site); President (BBB 'Business Management'); registered agent 'Johnson, Trish M' on the NC entity record (OpenCorporates us_nc/1154703)</t>
+          <t>Practice Owner</t>
         </is>
       </c>
       <c r="L11" s="8" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="BQ11" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: Compassionate Care Veterinary Hospital of Charlotte, P.A.. 1) Score is 65 QUALIFIED, call-first (D1 = 8: generic info@ only). Run the GEO spot-check (3 vet money questions x 2 platforms) — if she is named in 0 of 6, D4 = 10 and the row reaches 75 = SEND TODAY. 2) Build the voice demo from charlottepetdoctor.com (D2 = 15, demo_build = yes); script must route emergencies to Carolina Veterinary Specialists (704) 815-3939 / Skyline urgent care (704) 612-5590 immediately. 3) Not verified this run: Google rating/review count, owner reply behavior, Facebook/Instagram/X recency, LinkedIn, ads (Meta 403, Google Ads Transparency inconclusive), GBP hours — all blocked/JS-walled and WebSearch budget was exhausted mid-run. 4) GHL 'E4L Services' dedupe (ghl-contacts.js) not run — do it before load. 5) GeniusVets builds their site and sells vet SEO; the voice agent is the clean wedge, pitch GEO/website work second. 6) Hours conflict on their own site ('Monday - Thursday' vs 'CLOSED all day on Wednesdays') — treat Wednesday as closed; that line is also a safe, neutral opener. 7) Owner bio has personal/family detail — do not reference it; stick to her emergency-practice background, client-education focus, and the community drives. 8) Medical compliance: no promised outcomes, minimal health detail; the agent never triages. 9) BBB founding 1985 vs owner since 2007 suggests an acquired practice — unconfirmed; do not state it to her. 10) 1-DVM, 9-staff practice: Recover is first-fit but budget may push to the solo voice agent — no prices in email.</t>
+          <t>Title detail: Practice Owner and Veterinarian (site); President (BBB 'Business Management'); registered agent 'Johnson, Trish M' on the NC entity record (OpenCorporates us_nc/1154703). Legal entity note: legal: Compassionate Care Veterinary Hospital of Charlotte, P.A.. 1) Score is 65 QUALIFIED, call-first (D1 = 8: generic info@ only). Run the GEO spot-check (3 vet money questions x 2 platforms) — if she is named in 0 of 6, D4 = 10 and the row reaches 75 = SEND TODAY. 2) Build the voice demo from charlottepetdoctor.com (D2 = 15, demo_build = yes); script must route emergencies to Carolina Veterinary Specialists (704) 815-3939 / Skyline urgent care (704) 612-5590 immediately. 3) Not verified this run: Google rating/review count, owner reply behavior, Facebook/Instagram/X recency, LinkedIn, ads (Meta 403, Google Ads Transparency inconclusive), GBP hours — all blocked/JS-walled and WebSearch budget was exhausted mid-run. 4) GHL 'E4L Services' dedupe (ghl-contacts.js) not run — do it before load. 5) GeniusVets builds their site and sells vet SEO; the voice agent is the clean wedge, pitch GEO/website work second. 6) Hours conflict on their own site ('Monday - Thursday' vs 'CLOSED all day on Wednesdays') — treat Wednesday as closed; that line is also a safe, neutral opener. 7) Owner bio has personal/family detail — do not reference it; stick to her emergency-practice background, client-education focus, and the community drives. 8) Medical compliance: no promised outcomes, minimal health detail; the agent never triages. 9) BBB founding 1985 vs owner since 2007 suggests an acquired practice — unconfirmed; do not state it to her. 10) 1-DVM, 9-staff practice: Recover is first-fit but budget may push to the solo voice agent — no prices in email.</t>
         </is>
       </c>
       <c r="BR11" s="10" t="inlineStr"/>
@@ -8311,7 +8311,7 @@
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>President/CFO (BBB); 'one of the owners' in her own words on the Aurora Chamber listing</t>
+          <t>President/CFO</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
@@ -8601,7 +8601,7 @@
       </c>
       <c r="BQ12" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: U.B. Code Roofing Consultants, Inc.. Two decision-makers: Cynthia Smith (President/CFO, office, insurance paperwork, writes and signs replies, owns the named email) and Ronnie Smith (VP, "the owner" in the field, "50 years on roofs"). Email Cynthia; have Sam ask for either. Call window: Mountain Time, 7:00–8:30am or 4:00–5:30pm; main line +1 303-458-3790 (site number 303-225-4620 is likely Hibu tracking — fine to dial, but log which one Sam used). Incumbent: Hibu (site, likely ads/call tracking) + Podium (chat/text, reviews) — position the voice agent strictly as after-hours/overflow phone coverage that books into what they already use; do not pitch a site rebuild even though the About page still has lorem-ipsum placeholder copy (that is a later AI-readable-site conversation). Podium now sells AI phone answering — Sam should ask "who answers after 1pm Saturday right now?" on the first call and update D2 if Podium or an answering service is live. Email is Likely, not Confirmed (claimed Trustpilot profile, Oct 2025; MX present) — Rozel verify before send. Do not mention veteran status (BBB hints it; site only shows veteran discounts). Family-Legacy type: respect the 1998 / BBB-since-1999 history, slightly formal, no slang, no "AI" in the subject. GHL E4L Services dedupe (ghl-contacts.js) was not run from this session — run before load. D4 GEO audit not run (search budget exhausted) — run before send; this row cannot enter SEND TODAY until then. Google reviews/GBP hours were not opened directly; verify GBP hours match the site before quoting them on a call. HomeAdvisor says "Emergency services are not offered" while the site advertises emergency repair — do not quote either; just ask.</t>
+          <t>Title detail: President/CFO (BBB); 'one of the owners' in her own words on the Aurora Chamber listing. Legal entity note: legal: U.B. Code Roofing Consultants, Inc.. Two decision-makers: Cynthia Smith (President/CFO, office, insurance paperwork, writes and signs replies, owns the named email) and Ronnie Smith (VP, "the owner" in the field, "50 years on roofs"). Email Cynthia; have Sam ask for either. Call window: Mountain Time, 7:00–8:30am or 4:00–5:30pm; main line +1 303-458-3790 (site number 303-225-4620 is likely Hibu tracking — fine to dial, but log which one Sam used). Incumbent: Hibu (site, likely ads/call tracking) + Podium (chat/text, reviews) — position the voice agent strictly as after-hours/overflow phone coverage that books into what they already use; do not pitch a site rebuild even though the About page still has lorem-ipsum placeholder copy (that is a later AI-readable-site conversation). Podium now sells AI phone answering — Sam should ask "who answers after 1pm Saturday right now?" on the first call and update D2 if Podium or an answering service is live. Email is Likely, not Confirmed (claimed Trustpilot profile, Oct 2025; MX present) — Rozel verify before send. Do not mention veteran status (BBB hints it; site only shows veteran discounts). Family-Legacy type: respect the 1998 / BBB-since-1999 history, slightly formal, no slang, no "AI" in the subject. GHL E4L Services dedupe (ghl-contacts.js) was not run from this session — run before load. D4 GEO audit not run (search budget exhausted) — run before send; this row cannot enter SEND TODAY until then. Google reviews/GBP hours were not opened directly; verify GBP hours match the site before quoting them on a call. HomeAdvisor says "Emergency services are not offered" while the site advertises emergency repair — do not quote either; just ask.</t>
         </is>
       </c>
       <c r="BR12" s="10" t="inlineStr"/>
@@ -8652,7 +8652,7 @@
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>Owner (BBB 'Business Management: Cody Eason, Owner'; TN SOS registered agent at the LLC's head-office address per OpenCorporates; About-page photo caption 'Cody Eason - Hard at work'). Rutherford Chamber 'listed contact' NOT verifiable (page is JS-only). Second decision-maker: Jeremy Eason — 'Jeremy the owner was fantastic!' (Google review by 'Theo' on easonplumbing.com) and ProvenExpert contact person (no title). Cody PRIMARY (government + BBB), Jeremy LIKELY co-owner/family.</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
@@ -8942,7 +8942,7 @@
       </c>
       <c r="BQ13" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: EASON PLUMBING &amp; DRAIN CLEANING, LLC — TN SOS #001544246, Active. 1) Two Easons: Cody Eason is the legal/BBB owner (SOS registered agent, BBB 'Owner', Chamber contact); Jeremy Eason is called 'the owner' by a customer and is the ProvenExpert contact with jeremy@easonplumbing.com (LIKELY only — third-party directory; Rozel should flag Needs-Review before any send). Cody has no published email; office@ is CONFIRMED. Address them as a family team if unsure. 2) Band: 66 QUALIFIED, not SEND TODAY — D4 could not be run on ChatGPT/Perplexity/Gemini from this session; run the real GEO audit (no FAQPage schema; not named in 2 of 3 web-AI answers) and re-score; a '0 of 28' result plus the demo line likely lifts this into SEND TODAY. 3) Build the voice demo (D2 = 15, site scrapes cleanly; emergency page copy gives the 24/7 script). 4) Incumbent: Marketing 360 runs the site and tracking; the live placeholder on /get-a-quote/ suggests the relationship is neglected — raise it as a helpful observation, never as a dig at their vendor. 5) Not readable this session: Google reviews/reply behavior, Yelp owner section, Facebook posts, Meta Ad Library (403), Google Ads Transparency, TN license lookup (JS), Indeed (401) — Sam should log who answers and whether an answering service picks up after 5. 6) Hours conflict: site 7–5 Mon–Sat vs Yelp 'Open 24 hours' — ask on the call how after-hours calls are actually handled. 7) Suppression/seen checked clean; GHL 'E4L Services' dedupe by domain/phone was NOT run here — loader must run ghl-contacts.js before import. 8) Family-Legacy tone: slightly formal, reference the awards and 'three generations'; avoid 'modernize' language and avoid leading with 'AI'.</t>
+          <t>Title detail: Owner (BBB 'Business Management: Cody Eason, Owner'; TN SOS registered agent at the LLC's head-office address per OpenCorporates; About-page photo caption 'Cody Eason - Hard at work'). Rutherford Chamber 'listed contact' NOT verifiable (page is JS-only). Second decision-maker: Jeremy Eason — 'Jeremy the owner was fantastic!' (Google review by 'Theo' on easonplumbing.com) and ProvenExpert contact person (no title). Cody PRIMARY (government + BBB), Jeremy LIKELY co-owner/family.. Legal entity note: legal: EASON PLUMBING &amp; DRAIN CLEANING, LLC — TN SOS #001544246, Active. 1) Two Easons: Cody Eason is the legal/BBB owner (SOS registered agent, BBB 'Owner', Chamber contact); Jeremy Eason is called 'the owner' by a customer and is the ProvenExpert contact with jeremy@easonplumbing.com (LIKELY only — third-party directory; Rozel should flag Needs-Review before any send). Cody has no published email; office@ is CONFIRMED. Address them as a family team if unsure. 2) Band: 66 QUALIFIED, not SEND TODAY — D4 could not be run on ChatGPT/Perplexity/Gemini from this session; run the real GEO audit (no FAQPage schema; not named in 2 of 3 web-AI answers) and re-score; a '0 of 28' result plus the demo line likely lifts this into SEND TODAY. 3) Build the voice demo (D2 = 15, site scrapes cleanly; emergency page copy gives the 24/7 script). 4) Incumbent: Marketing 360 runs the site and tracking; the live placeholder on /get-a-quote/ suggests the relationship is neglected — raise it as a helpful observation, never as a dig at their vendor. 5) Not readable this session: Google reviews/reply behavior, Yelp owner section, Facebook posts, Meta Ad Library (403), Google Ads Transparency, TN license lookup (JS), Indeed (401) — Sam should log who answers and whether an answering service picks up after 5. 6) Hours conflict: site 7–5 Mon–Sat vs Yelp 'Open 24 hours' — ask on the call how after-hours calls are actually handled. 7) Suppression/seen checked clean; GHL 'E4L Services' dedupe by domain/phone was NOT run here — loader must run ghl-contacts.js before import. 8) Family-Legacy tone: slightly formal, reference the awards and 'three generations'; avoid 'modernize' language and avoid leading with 'AI'.</t>
         </is>
       </c>
       <c r="BR13" s="10" t="inlineStr"/>
@@ -8993,7 +8993,7 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>Co-owner / co-founder (Marlin "Scott" Clark Sr.); co-owner Glenda Clark (bought her father's half in 2006, handles accounting); Marlin Clark Jr. 3rd generation (joined 2016) and registered agent of record</t>
+          <t>Co-owner / co-founder</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -9283,7 +9283,7 @@
       </c>
       <c r="BQ14" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: MARLIN JAMES INC., FL doc # P97000034717, Active; license CAC056868 per site. Second decision-maker: Glenda Clark (co-owner; "My father's only stipulation was that I do the accounting" — likely signs the checks). Next-gen champion: Marlin Clark Jr. (joined 2016, registered agent of record) — per the Family-Legacy playbook, consider addressing him and copying Scott/Glenda. Gatekeeper: Shannon Gluch, maintenance coordinator (company spokesperson in the Oct 2025 article). Tone: warm, slightly formal, no slang; the brand makes faith-forward statements on its own site ("serve... with a servant's heart") — brand-level only, mirror respect for the legacy and never lead with "AI"; position the agent as after-hours/overflow only, never as replacing office staff. They run ServiceTitan (Text2Chat widget key in source) — say "books into ServiceTitan" and do not pitch chat/text. No email anywhere → DEMO PATH / Sam call; best window trades 7:00-8:30am or 4:00-5:30pm ET, inside office hours 8-5 M-F; Florida calling window is 8am-8pm and Florida has a mini-TCPA/telemarketer-registration rule — confirm before Sam dials; the main number is advertised as "call or text" so treat it as a possible cell: manual dial only, no SMS or AI voice. Yelp 3.5 on 11 vs Google 4.8 on 368 — Yelp blocked this run, read the lows by hand before the call and never quote a negative review. AI spot-check not run (search budget) and GHL dedupe (ghl-contacts.js) not run — do both before loading or emailing. Founder "Red" Griffin is listed on the site as 1944-2018; reference Red's Club and WWRD, not the founder's passing. Sunbiz (403) and DBPR CAC056868 (error page) could not be read; entity status Active via OpenCorporates P97000034717 — spot-check Sunbiz by hand if the deal progresses. Local-media relationship with Osprey Observer (features 2019, 2024, 2025; podcast Jul 2024) — they like telling the story on record</t>
+          <t>Title detail: Co-owner / co-founder (Marlin "Scott" Clark Sr.); co-owner Glenda Clark (bought her father's half in 2006, handles accounting); Marlin Clark Jr. 3rd generation (joined 2016) and registered agent of record. Legal entity note: legal: MARLIN JAMES INC., FL doc # P97000034717, Active; license CAC056868 per site. Second decision-maker: Glenda Clark (co-owner; "My father's only stipulation was that I do the accounting" — likely signs the checks). Next-gen champion: Marlin Clark Jr. (joined 2016, registered agent of record) — per the Family-Legacy playbook, consider addressing him and copying Scott/Glenda. Gatekeeper: Shannon Gluch, maintenance coordinator (company spokesperson in the Oct 2025 article). Tone: warm, slightly formal, no slang; the brand makes faith-forward statements on its own site ("serve... with a servant's heart") — brand-level only, mirror respect for the legacy and never lead with "AI"; position the agent as after-hours/overflow only, never as replacing office staff. They run ServiceTitan (Text2Chat widget key in source) — say "books into ServiceTitan" and do not pitch chat/text. No email anywhere → DEMO PATH / Sam call; best window trades 7:00-8:30am or 4:00-5:30pm ET, inside office hours 8-5 M-F; Florida calling window is 8am-8pm and Florida has a mini-TCPA/telemarketer-registration rule — confirm before Sam dials; the main number is advertised as "call or text" so treat it as a possible cell: manual dial only, no SMS or AI voice. Yelp 3.5 on 11 vs Google 4.8 on 368 — Yelp blocked this run, read the lows by hand before the call and never quote a negative review. AI spot-check not run (search budget) and GHL dedupe (ghl-contacts.js) not run — do both before loading or emailing. Founder "Red" Griffin is listed on the site as 1944-2018; reference Red's Club and WWRD, not the founder's passing. Sunbiz (403) and DBPR CAC056868 (error page) could not be read; entity status Active via OpenCorporates P97000034717 — spot-check Sunbiz by hand if the deal progresses. Local-media relationship with Osprey Observer (features 2019, 2024, 2025; podcast Jul 2024) — they like telling the story on record</t>
         </is>
       </c>
       <c r="BR14" s="10" t="inlineStr"/>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>Owner (site: "assume ownership", Feb 2017) / President/CEO (BBB Business Management: "Casey M. Tynan")</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="L15" s="8" t="inlineStr">
@@ -9624,7 +9624,7 @@
       </c>
       <c r="BQ15" s="8" t="inlineStr">
         <is>
-          <t>1) Entity flag for Rozel: the Colorado corp EFFICIENCY GARAGE DOOR SERVICE, INC. (#19871530966, Bob Hershey era) was voluntarily dissolved 2017-12-19 — consistent with Casey buying the business Feb 2017 and the old owner winding up his corporation; the current operating entity's name was NOT FOUND (CO SOS blocked by Cloudflare; OpenCorporates searches for "Efficiency Garage Door" and "EGDS" show only the dissolved corp). The business is demonstrably live (site edited 2026-09-01, BBB A+ accredited, 0 complaints) so this is not treated as a disqualifier, but confirm before loading. 2) Not run this session: GHL 'E4L Services' dedupe (ghl-contacts.js), Google Business Profile (rating, hours, reviews, reply rate), Yelp (403), Indeed (403), Meta Ad Library / Google Ads Transparency / LSA, and the D4 AI spot-check — the WebSearch budget was exhausted; score is PROVISIONAL at 62 until these are filled. 3) Email is CONFIRMED (own site, 4 pages, MX present) — safe for Sebastian's plain-text cold email; no secondary channel, so Sam's call is the second touch. 4) Opener-safe facts: 1963 founding, Bob Hershey's 50 years, Casey's Feb 2017 takeover, the hours-vs-emergency gap, no online scheduler. Do NOT mention the lorem-ipsum blog posts or the dissolved corp in outreach. 5) Attitude is Family-Legacy; keep tone slightly formal, no "disrupt/modernize," position voice AI as after-hours/overflow only. 6) Not previously demoed or audited (no egds mention in geo/audits or lead-machine data; not on suppression.csv or seen.csv).</t>
+          <t>Title detail: Owner (site: "assume ownership", Feb 2017) / President/CEO (BBB Business Management: "Casey M. Tynan"). 1) Entity flag for Rozel: the Colorado corp EFFICIENCY GARAGE DOOR SERVICE, INC. (#19871530966, Bob Hershey era) was voluntarily dissolved 2017-12-19 — consistent with Casey buying the business Feb 2017 and the old owner winding up his corporation; the current operating entity's name was NOT FOUND (CO SOS blocked by Cloudflare; OpenCorporates searches for "Efficiency Garage Door" and "EGDS" show only the dissolved corp). The business is demonstrably live (site edited 2026-09-01, BBB A+ accredited, 0 complaints) so this is not treated as a disqualifier, but confirm before loading. 2) Not run this session: GHL 'E4L Services' dedupe (ghl-contacts.js), Google Business Profile (rating, hours, reviews, reply rate), Yelp (403), Indeed (403), Meta Ad Library / Google Ads Transparency / LSA, and the D4 AI spot-check — the WebSearch budget was exhausted; score is PROVISIONAL at 62 until these are filled. 3) Email is CONFIRMED (own site, 4 pages, MX present) — safe for Sebastian's plain-text cold email; no secondary channel, so Sam's call is the second touch. 4) Opener-safe facts: 1963 founding, Bob Hershey's 50 years, Casey's Feb 2017 takeover, the hours-vs-emergency gap, no online scheduler. Do NOT mention the lorem-ipsum blog posts or the dissolved corp in outreach. 5) Attitude is Family-Legacy; keep tone slightly formal, no "disrupt/modernize," position voice AI as after-hours/overflow only. 6) Not previously demoed or audited (no egds mention in geo/audits or lead-machine data; not on suppression.csv or seen.csv).</t>
         </is>
       </c>
       <c r="BR15" s="10" t="inlineStr"/>
@@ -9675,7 +9675,7 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>Orthodontist, DDS, MSD - leads the practice ("Led by... Dr. Fowler", "one-doctor, one-location practice"); registered agent of FOWLER ORTHODONTICS, PLLC as "CHAD E FOWLER" at the practice address. Explicit "owner" title not stated on site; OpenCorporates shows "1 officer" behind login.</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -9965,7 +9965,7 @@
       </c>
       <c r="BQ16" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: FOWLER ORTHODONTICS, PLLC, TN control #000549400, status Active. Email route: drfowler@fowlerortho.com is the published resume inbox, so he reads it personally; keep the subject clearly non-recruiting so it isn't filed as an application. Call window: Tue-Thu 10am-12pm Central (office closed Fridays per site). Gatekeeper: the form page references a "scheduling coordinator" (no names found; no team page). Second decision-maker: none found. Incumbent: Sesame Communications (web + likely reminders/portal) - do not open with a website rebuild; Ortho2 is the practice-management system (online forms), so "books into your Ortho2 schedule" is the integration question to be ready for. Compliance: medical vertical - no promised results, keep health detail minimal; do not mention the 2015 Haiti mission or hobbies beyond a light touch. GEO audit set: Healthgrades shows 28 orthodontists within 10 miles. NOT CHECKED this run (log for Rozel): Google review count/rating and owner reply rate (Maps not fetchable), LinkedIn (search budget exhausted), Meta Ad Library/Google Ads/LSA, AI spot-check, TN SOS detail (503 x2 - OpenCorporates mirror used), Yelp (403), Instagram (429), Facebook (login wall), Wayback (egress blocked). Dedupe: suppression.csv clear; GHL 'E4L Services' dedupe still required before load.</t>
+          <t>Title detail: Orthodontist, DDS, MSD - leads the practice ("Led by... Dr. Fowler", "one-doctor, one-location practice"); registered agent of FOWLER ORTHODONTICS, PLLC as "CHAD E FOWLER" at the practice address. Explicit "owner" title not stated on site; OpenCorporates shows "1 officer" behind login.. Legal entity note: legal: FOWLER ORTHODONTICS, PLLC, TN control #000549400, status Active. Email route: drfowler@fowlerortho.com is the published resume inbox, so he reads it personally; keep the subject clearly non-recruiting so it isn't filed as an application. Call window: Tue-Thu 10am-12pm Central (office closed Fridays per site). Gatekeeper: the form page references a "scheduling coordinator" (no names found; no team page). Second decision-maker: none found. Incumbent: Sesame Communications (web + likely reminders/portal) - do not open with a website rebuild; Ortho2 is the practice-management system (online forms), so "books into your Ortho2 schedule" is the integration question to be ready for. Compliance: medical vertical - no promised results, keep health detail minimal; do not mention the 2015 Haiti mission or hobbies beyond a light touch. GEO audit set: Healthgrades shows 28 orthodontists within 10 miles. NOT CHECKED this run (log for Rozel): Google review count/rating and owner reply rate (Maps not fetchable), LinkedIn (search budget exhausted), Meta Ad Library/Google Ads/LSA, AI spot-check, TN SOS detail (503 x2 - OpenCorporates mirror used), Yelp (403), Instagram (429), Facebook (login wall), Wayback (egress blocked). Dedupe: suppression.csv clear; GHL 'E4L Services' dedupe still required before load.</t>
         </is>
       </c>
       <c r="BR16" s="10" t="inlineStr"/>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>President / Managing Member (BBB principal: "James A. Adams, President/Managing Member"); Master Electrician (site: "Master Electrician James Adams"; TDLR Master Electrician #220484, TECL #27762 on site); registered agent of ABR Electric LLC (OpenCorporates)</t>
+          <t>President / Managing Member</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
@@ -10302,7 +10302,7 @@
       </c>
       <c r="BQ17" s="8" t="inlineStr">
         <is>
-          <t>1) Route: DEMO PATH / call-first — no email anywhere public (MX exists, so a mailbox is unpublished; do not pattern-guess). Build the voice demo from abrelectric.com before Sam's call. 2) D4 not run: the AI spot-check and ad-library checks were impossible this session (search budget exhausted; GBP/Yelp/Facebook/LinkedIn/Indeed/ad libraries unfetchable). Run the GEO audit before quoting any "Named in X of Y" line. 3) Caution: robots.txt on their site disallows an "/AI/" path titled "Private AI &amp; SEO Reports" — they (or a web vendor) already monitor AI/SEO visibility. I only saw the public index title and did not go further; do not reference it in outreach, and expect James to already understand GEO. 4) Hours conflict: site says 7AM–7PM; a Google-listing-sourced directory says 8AM–4PM — if the Google listing is right, the evening gap is bigger than the site implies; Sam can confirm by what answers at 5 PM. 5) Owner profile: veteran-owned ("Airborne Ranger" on the About page), Master Electrician, YouTube educator (11.9K subs, 432 videos), teaches licensing workshops, publishes prices — pragmatic, proof-driven, anti-hype; lead with the demo number, no hype words, no "AI" in the subject line. 6) Second decision-maker: Nathan Tiner, COO (BBB) — hands-on with quotes per a site review; Cynthia E. Adams is Managing Member (business record only). Gatekeeper: "Wendy in the office" (customer review on their site). 7) Entity: ABR Electric LLC formed 2021-11-23 (TX co. 0804324904) vs BBB "started 2010" — CONFLICT, likely reorg from the older inactive A B R Electric, Inc.; the Plano registered-agent address on OpenCorporates may be residential — not recorded. 8) GHL "E4L Services" dedupe (ghl-contacts.js by domain/phone/name+city) was not run in this session — run before loading. 9) They appear in serviceagent.ai's directory (an AI-receptionist vendor), so they have likely been pitched by competitors — differentiate on the pre-paid live demo built from their own site and the one-rule go-live/rollback. 10) Compliance: main line is "call or text" per BBB but no SMS consent exists — manual dial only.</t>
+          <t>Title detail: President / Managing Member (BBB principal: "James A. Adams, President/Managing Member"); Master Electrician (site: "Master Electrician James Adams"; TDLR Master Electrician #220484, TECL #27762 on site); registered agent of ABR Electric LLC (OpenCorporates). 1) Route: DEMO PATH / call-first — no email anywhere public (MX exists, so a mailbox is unpublished; do not pattern-guess). Build the voice demo from abrelectric.com before Sam's call. 2) D4 not run: the AI spot-check and ad-library checks were impossible this session (search budget exhausted; GBP/Yelp/Facebook/LinkedIn/Indeed/ad libraries unfetchable). Run the GEO audit before quoting any "Named in X of Y" line. 3) Caution: robots.txt on their site disallows an "/AI/" path titled "Private AI &amp; SEO Reports" — they (or a web vendor) already monitor AI/SEO visibility. I only saw the public index title and did not go further; do not reference it in outreach, and expect James to already understand GEO. 4) Hours conflict: site says 7AM–7PM; a Google-listing-sourced directory says 8AM–4PM — if the Google listing is right, the evening gap is bigger than the site implies; Sam can confirm by what answers at 5 PM. 5) Owner profile: veteran-owned ("Airborne Ranger" on the About page), Master Electrician, YouTube educator (11.9K subs, 432 videos), teaches licensing workshops, publishes prices — pragmatic, proof-driven, anti-hype; lead with the demo number, no hype words, no "AI" in the subject line. 6) Second decision-maker: Nathan Tiner, COO (BBB) — hands-on with quotes per a site review; Cynthia E. Adams is Managing Member (business record only). Gatekeeper: "Wendy in the office" (customer review on their site). 7) Entity: ABR Electric LLC formed 2021-11-23 (TX co. 0804324904) vs BBB "started 2010" — CONFLICT, likely reorg from the older inactive A B R Electric, Inc.; the Plano registered-agent address on OpenCorporates may be residential — not recorded. 8) GHL "E4L Services" dedupe (ghl-contacts.js by domain/phone/name+city) was not run in this session — run before loading. 9) They appear in serviceagent.ai's directory (an AI-receptionist vendor), so they have likely been pitched by competitors — differentiate on the pre-paid live demo built from their own site and the one-rule go-live/rollback. 10) Compliance: main line is "call or text" per BBB but no SMS consent exists — manual dial only.</t>
         </is>
       </c>
       <c r="BR17" s="10" t="inlineStr"/>
@@ -10353,7 +10353,7 @@
       </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>Owner (BBB "Business Management": Abraham Valentin, Owner). Second decision-maker: Lelia Valentin, President (BBB) — corroborated as "LELIA M VALENTIN", registered agent of ABE'S ELECTRIC INC at 1004 Royal Street (Florida Sunbiz record via OpenCorporates). On-site Google reviews mention "Lisa and Abe" — recorded as-is, NOT reconciled with Lelia.</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="L18" s="8" t="inlineStr">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="BQ18" s="8" t="inlineStr">
         <is>
-          <t>Route: call-first (D1 = 8, generic mailbox only) per rubric; Sam calls Tue–Thu 8:00–8:30 AM ET and asks for Abe (or Lisa for the office side); an email to contact@abeselectric.com addressed to Abe and Lelia is the secondary touch. Do not call before 8:00 AM ET (Florida 8–8 rule). Pre-build the demo line from abeselectric.com (phone-first, D2 = 15). Run the D4 AI spot-check before any "Named in X of Y" claim — it was not run this run. GHL "E4L Services" dedupe was NOT run in this session (only suppression.csv/seen.csv were checked) — run it before loading. Reviews, GBP hours/replies, Facebook, Instagram, Yelp, Indeed, Wayback and ad libraries were all unreachable this run, so review-reply tone and ad spend are unknown; Sam should log who/what answers the line. Site reviews say "Lisa and Abe"; BBB says Lelia Valentin, President — never assume they are the same person. The site was built on Lovable (an AI site builder), so the team is comfortable with new tools, but the homepage's "real person, not a call center" line means keep "AI" out of the subject line and lead with after-hours coverage. Founding-year CONFLICT (domain 2001, BBB 2007, current FL entity 2020 with older inactive entities) — use "since 2007" only softly or not at all. Older BBB address (886 Duncan Ave) and 877 number may be legacy; use 1004 Royal St and (407) 343-0220.</t>
+          <t>Title detail: Owner (BBB "Business Management": Abraham Valentin, Owner). Second decision-maker: Lelia Valentin, President (BBB) — corroborated as "LELIA M VALENTIN", registered agent of ABE'S ELECTRIC INC at 1004 Royal Street (Florida Sunbiz record via OpenCorporates). On-site Google reviews mention "Lisa and Abe" — recorded as-is, NOT reconciled with Lelia.. Route: call-first (D1 = 8, generic mailbox only) per rubric; Sam calls Tue–Thu 8:00–8:30 AM ET and asks for Abe (or Lisa for the office side); an email to contact@abeselectric.com addressed to Abe and Lelia is the secondary touch. Do not call before 8:00 AM ET (Florida 8–8 rule). Pre-build the demo line from abeselectric.com (phone-first, D2 = 15). Run the D4 AI spot-check before any "Named in X of Y" claim — it was not run this run. GHL "E4L Services" dedupe was NOT run in this session (only suppression.csv/seen.csv were checked) — run it before loading. Reviews, GBP hours/replies, Facebook, Instagram, Yelp, Indeed, Wayback and ad libraries were all unreachable this run, so review-reply tone and ad spend are unknown; Sam should log who/what answers the line. Site reviews say "Lisa and Abe"; BBB says Lelia Valentin, President — never assume they are the same person. The site was built on Lovable (an AI site builder), so the team is comfortable with new tools, but the homepage's "real person, not a call center" line means keep "AI" out of the subject line and lead with after-hours coverage. Founding-year CONFLICT (domain 2001, BBB 2007, current FL entity 2020 with older inactive entities) — use "since 2007" only softly or not at all. Older BBB address (886 Duncan Ave) and 877 number may be legacy; use 1004 Royal St and (407) 343-0220.</t>
         </is>
       </c>
       <c r="BR18" s="10" t="inlineStr"/>
@@ -10694,7 +10694,7 @@
       </c>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>Owner / Board Chair (site: "Dave Turner Owner/Board Chair", https://www.flobeds.com/about-us/); BBB lists "Mr. David R. Turner, President" (https://www.bbb.org/us/ca/fort-bragg/profile/mattress/flobeds-1116-15241). Day-to-day President is Dewey Turner (site), ~15 years in the family business.</t>
+          <t>Owner / Board Chair</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
@@ -10984,7 +10984,7 @@
       </c>
       <c r="BQ19" s="8" t="inlineStr">
         <is>
-          <t>Address the email to Dewey Turner (President, day-to-day, personally answers service emails per a Nov 2025 review) and mention Dave by name; Anne Turner (Owner/VP, bookkeeper) likely sees any invoice. Only generic mailboxes exist (info@, service@) — send to info@ with "For Dewey" in the first line, and have Sam call 1-800-356-2337 and ask for Dewey by name; best window Tue–Thu 9–11am PT (live person 8–5 PT; avoid Saturday). Do not quote the 2018/2021 email complaints back to them — summarize as "a couple of older reviews." Flags for Rozel: CA SOS entity status not confirmed (API blocked; OpenCorporates 0 hits under "flobeds" — legal name may differ); GHL dedupe not run; founding year CONFLICT 1971 vs 1989; blog byline "Jacob Taylor" could be an in-house marketing/content person — verify before pitching the content engine; D4 AI spot-check must be run before any SEND TODAY promotion (search budget exhausted this session); Google rating/GBP not retrieved. Compliance: not a medical vertical, but never imply sleep/health outcomes from a mattress in copy. Local color: Fort Bragg's Paul Bunyan Days (Labor Day weekend) — FloBeds built the "world's largest dog bed" there in 2010. BBB-listed phone (707) 964-3356 differs from the two website numbers.</t>
+          <t>Title detail: Owner / Board Chair (site: "Dave Turner Owner/Board Chair", https://www.flobeds.com/about-us/); BBB lists "Mr. David R. Turner, President" (https://www.bbb.org/us/ca/fort-bragg/profile/mattress/flobeds-1116-15241). Day-to-day President is Dewey Turner (site), ~15 years in the family business.. Address the email to Dewey Turner (President, day-to-day, personally answers service emails per a Nov 2025 review) and mention Dave by name; Anne Turner (Owner/VP, bookkeeper) likely sees any invoice. Only generic mailboxes exist (info@, service@) — send to info@ with "For Dewey" in the first line, and have Sam call 1-800-356-2337 and ask for Dewey by name; best window Tue–Thu 9–11am PT (live person 8–5 PT; avoid Saturday). Do not quote the 2018/2021 email complaints back to them — summarize as "a couple of older reviews." Flags for Rozel: CA SOS entity status not confirmed (API blocked; OpenCorporates 0 hits under "flobeds" — legal name may differ); GHL dedupe not run; founding year CONFLICT 1971 vs 1989; blog byline "Jacob Taylor" could be an in-house marketing/content person — verify before pitching the content engine; D4 AI spot-check must be run before any SEND TODAY promotion (search budget exhausted this session); Google rating/GBP not retrieved. Compliance: not a medical vertical, but never imply sleep/health outcomes from a mattress in copy. Local color: Fort Bragg's Paul Bunyan Days (Labor Day weekend) — FloBeds built the "world's largest dog bed" there in 2010. BBB-listed phone (707) 964-3356 differs from the two website numbers.</t>
         </is>
       </c>
       <c r="BR19" s="10" t="inlineStr"/>
@@ -11031,7 +11031,7 @@
       <c r="J20" s="8" t="inlineStr"/>
       <c r="K20" s="8" t="inlineStr">
         <is>
-          <t>Founder / "matriarch" (About page; surname not published anywhere found). Family decision-makers also cited: Jana Marcelino — listed in BBB profile structured data as "Mrs. Jana Marcelino" (employee; no title shown) and LIKELY the daughter "Jana" named on About; Dannielli Marcelino, RN — master injector (LinkedIn company People tab + About "Dannielli RN"); Jeanie — Medical Consultant (About); Saharra — granddaughter, laser tech (About).</t>
+          <t>Founder / "matriarch"</t>
         </is>
       </c>
       <c r="L20" s="8" t="inlineStr">
@@ -11321,7 +11321,7 @@
       </c>
       <c r="BQ20" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal owner per site privacy policy: Zen Garden Enterprises, LLC — AZ L12735933. DECISION-MAKERS: three-generation family. Founder Luzivone (surname never published — do not guess; the retail line "Marcelino MD" and daughters' surname Marcelino on BBB/LinkedIn do NOT establish hers). Best names to ask for: Jana Marcelino (BBB lists "Mrs. Jana Marcelino" in its business record, title not shown — LIKELY the daughter "Jana" on About) and Dannielli Marcelino, RN (master injector, the face of the clinical side and the TikTok/promo content). Jeanie = "Medical Consultant"; granddaughter Saharra = laser tech with TV appearances (possible next-gen champion per the Family-Legacy playbook). Medical Director Dr. Brit Ferrell MD is not the buyer. LEGAL: privacy policy says the site is "owned and operated by Zen Garden Enterprises" — OpenCorporates shows ZEN GARDEN ENTERPRISES, LLC (AZ L12735933, Active, Articles of Organization 2006-03-28, agent Document Prep &amp; Process Pros, 3 officers behind login). ecorp.azcc.gov was unreachable from this sandbox — have Abdullah pull the member names there (2 minutes) to upgrade D1. Old entity Suddenly Slimmer, Inc. (08732090) dissolved 2004-01-13. GATEKEEPER: front desk "spa coordinators" (per hiring page). CALL WINDOW: Tue–Thu 10am–12pm Arizona time (AZ has no DST: same as LA through Oct 31, then 9–11am LA from Nov 1). PHONE: main +1 602-952-8446 is "call or text" — human manual dial only; the second number 602-737-1788 behind the mobile Call button is unexplained — leave it alone. COMPLIANCE: medical — never promise results, never quote treatment prices (their site lists per-unit Botox pricing; don't echo it). Don't mention the BBB C+ / 4 complaints. Hiring page is evergreen (2023) — don't say "saw you're hiring this week." GEO PITCH NUANCE: site already carries LocalBusiness/Organization JSON-LD and a 6-question FAQPage schema, so pitch answer-page content and money-question coverage, not "we'll add schema." Run the full 28-answer audit before any touch (Truth-in-offers rule — no "Named in X of 28" line exists yet). GAPS THIS RUN: web search budget hit, so Google reviews, Yelp (403), Instagram (429), Meta Ad Library (403), Google LSA and AI spot-checks were not readable; Wayback CDX returned nothing. Suppression: clean. Case-study proximity: E4L has an existing med spa client and GEO template — worth citing on the call.</t>
+          <t>Title detail: Founder / "matriarch" (About page; surname not published anywhere found). Family decision-makers also cited: Jana Marcelino — listed in BBB profile structured data as "Mrs. Jana Marcelino" (employee; no title shown) and LIKELY the daughter "Jana" named on About; Dannielli Marcelino, RN — master injector (LinkedIn company People tab + About "Dannielli RN"); Jeanie — Medical Consultant (About); Saharra — granddaughter, laser tech (About).. Legal entity note: legal owner per site privacy policy: Zen Garden Enterprises, LLC — AZ L12735933. DECISION-MAKERS: three-generation family. Founder Luzivone (surname never published — do not guess; the retail line "Marcelino MD" and daughters' surname Marcelino on BBB/LinkedIn do NOT establish hers). Best names to ask for: Jana Marcelino (BBB lists "Mrs. Jana Marcelino" in its business record, title not shown — LIKELY the daughter "Jana" on About) and Dannielli Marcelino, RN (master injector, the face of the clinical side and the TikTok/promo content). Jeanie = "Medical Consultant"; granddaughter Saharra = laser tech with TV appearances (possible next-gen champion per the Family-Legacy playbook). Medical Director Dr. Brit Ferrell MD is not the buyer. LEGAL: privacy policy says the site is "owned and operated by Zen Garden Enterprises" — OpenCorporates shows ZEN GARDEN ENTERPRISES, LLC (AZ L12735933, Active, Articles of Organization 2006-03-28, agent Document Prep &amp; Process Pros, 3 officers behind login). ecorp.azcc.gov was unreachable from this sandbox — have Abdullah pull the member names there (2 minutes) to upgrade D1. Old entity Suddenly Slimmer, Inc. (08732090) dissolved 2004-01-13. GATEKEEPER: front desk "spa coordinators" (per hiring page). CALL WINDOW: Tue–Thu 10am–12pm Arizona time (AZ has no DST: same as LA through Oct 31, then 9–11am LA from Nov 1). PHONE: main +1 602-952-8446 is "call or text" — human manual dial only; the second number 602-737-1788 behind the mobile Call button is unexplained — leave it alone. COMPLIANCE: medical — never promise results, never quote treatment prices (their site lists per-unit Botox pricing; don't echo it). Don't mention the BBB C+ / 4 complaints. Hiring page is evergreen (2023) — don't say "saw you're hiring this week." GEO PITCH NUANCE: site already carries LocalBusiness/Organization JSON-LD and a 6-question FAQPage schema, so pitch answer-page content and money-question coverage, not "we'll add schema." Run the full 28-answer audit before any touch (Truth-in-offers rule — no "Named in X of 28" line exists yet). GAPS THIS RUN: web search budget hit, so Google reviews, Yelp (403), Instagram (429), Meta Ad Library (403), Google LSA and AI spot-checks were not readable; Wayback CDX returned nothing. Suppression: clean. Case-study proximity: E4L has an existing med spa client and GEO template — worth citing on the call.</t>
         </is>
       </c>
       <c r="BR20" s="10" t="inlineStr"/>
@@ -11372,7 +11372,7 @@
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>Owner / NC Heating Contractor license holder (Groups 1, 2, 3) — LinkedIn headline 'Small Business Owner'; Yelp 'Business Owner'; NC Board record lists 'Contact Name: Robert Allen George' for AirPro Carolina, LLC; OpenCorporates registered agent 'George, Robert Allen'; Google Ads verified advertiser legal name 'Robert A George'</t>
+          <t>Owner / NC Heating Contractor license holder</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
@@ -11662,7 +11662,7 @@
       </c>
       <c r="BQ21" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal entity: AirPro Carolina, LLC. 1) Owner is nailed down: Robert Allen 'Rob' George — NC Board license L.32262 lists him as contact and sole classification holder for AirPro Carolina, LLC at the business address/phone; he is also the registered agent and the verified Google Ads advertiser. Use 'Rob'. 2) Route call-first: only a generic info@ exists (and only inside the site's JSON-LD). Email as a second touch at most; keep it plain-text, no links. 3) Hours conflict is the whole pitch: site says Mon–Fri 8–5 with after-hours 'based on technician availability'; GBP says 'Open 24 hours'. After-hours calls are billed at a premium internally — do not quote their pricing back to him. 4) Incumbent caveat: 'Powered by Unify360' on the site — that vendor sells AI text/chat/form/LSA lead response + reputation + lead management. Only the review widget is confirmed; chat is Tidio. Ask on the call whether anything answers the phone after hours; if Unify360's AI agent is live on texts/chats, pivot to voice-only + GEO. 5) D4 not run (all AI platforms bot-blocked here) — run the full GEO audit before any email so the 'Named in X of 28' line is real; site has HVACBusiness schema but no FAQPage. 6) Tech-forward, no-hype owner: name his stack (Housecall Pro, Tidio, Google Ads), keep it short, lead with the demo number, never promise results. 7) Safe warm compliments: the animal-rescue work (feral-cat TNR, No Empty Bowl Project) and the Oct 4 heating-season post. 8) Score 61 / TRUSTED / QUALIFIED; would rise to 65+ if a live Google Sponsored result is observed (D6 → 15). Phone discrepancy: ignore (919) 582-5022 unless 578-7798 fails.</t>
+          <t>Title detail: Owner / NC Heating Contractor license holder (Groups 1, 2, 3) — LinkedIn headline 'Small Business Owner'; Yelp 'Business Owner'; NC Board record lists 'Contact Name: Robert Allen George' for AirPro Carolina, LLC; OpenCorporates registered agent 'George, Robert Allen'; Google Ads verified advertiser legal name 'Robert A George'. Legal entity note: legal entity: AirPro Carolina, LLC. 1) Owner is nailed down: Robert Allen 'Rob' George — NC Board license L.32262 lists him as contact and sole classification holder for AirPro Carolina, LLC at the business address/phone; he is also the registered agent and the verified Google Ads advertiser. Use 'Rob'. 2) Route call-first: only a generic info@ exists (and only inside the site's JSON-LD). Email as a second touch at most; keep it plain-text, no links. 3) Hours conflict is the whole pitch: site says Mon–Fri 8–5 with after-hours 'based on technician availability'; GBP says 'Open 24 hours'. After-hours calls are billed at a premium internally — do not quote their pricing back to him. 4) Incumbent caveat: 'Powered by Unify360' on the site — that vendor sells AI text/chat/form/LSA lead response + reputation + lead management. Only the review widget is confirmed; chat is Tidio. Ask on the call whether anything answers the phone after hours; if Unify360's AI agent is live on texts/chats, pivot to voice-only + GEO. 5) D4 not run (all AI platforms bot-blocked here) — run the full GEO audit before any email so the 'Named in X of 28' line is real; site has HVACBusiness schema but no FAQPage. 6) Tech-forward, no-hype owner: name his stack (Housecall Pro, Tidio, Google Ads), keep it short, lead with the demo number, never promise results. 7) Safe warm compliments: the animal-rescue work (feral-cat TNR, No Empty Bowl Project) and the Oct 4 heating-season post. 8) Score 61 / TRUSTED / QUALIFIED; would rise to 65+ if a live Google Sponsored result is observed (D6 → 15). Phone discrepancy: ignore (919) 582-5022 unless 578-7798 fails.</t>
         </is>
       </c>
       <c r="BR21" s="10" t="inlineStr"/>
@@ -11713,7 +11713,7 @@
       </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>Owner / Member (BBB Business Management) and AZ ROC Qualifying Party (BuildZoom); customers call him 'the owner Josh'; Apr-2024 press release calls him 'founder and CEO'</t>
+          <t>Owner / Member</t>
         </is>
       </c>
       <c r="L22" s="8" t="inlineStr">
@@ -12003,7 +12003,7 @@
       </c>
       <c r="BQ22" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: MOREHART AIR CONDITIONING AND HEATING LLC, AZ entity L14058381. (1) Route: DEMO PATH / call-first - no email exists publicly; Sam dials, asks for Josh by name; owner title on record is "Member" (BBB), he is the ROC qualifying party and works in the field. (2) Second decision-maker: Janah M Morehart, Member and registered agent (BBB details; OpenCorporates) - co-owner on record, treat as co-signer. (3) Champion/gatekeeper: Mayley Madrid, Business Development Coordinator (BBB) - praised in a site review for coordinating a same-day after-hours dispatch ("communicated with us while she worked on getting Thomas out"), so she likely owns the phone process; position the AI as after-hours/overflow only, never as replacing her. Also on record: Jeremy Robert Grubbs, Qp/Member (BuildZoom ROC-derived). Long-tenured tech Brian Sturgeon (14 yrs per a reviewer). (4) Phones: 602-640-0444 is site-only (likely RYNO tracking number, GTM present); 623-566-0005 is the number in their schema, BBB, and press - dial 623 for the office, dial 602 once after 5pm MST to hear what the tracked line actually does. Arizona has no DST (MST, UTC-7); trades window 7:00-8:30am or 4:00-5:30pm local. (5) They already collect TCPA-style SMS consent on every form, so missed-call text-back slots into an existing habit. (6) Incumbent: RYNO Strategic Solutions (HVAC-vertical web/marketing) - do not pitch web; phone + GEO wedge only; site has HVACBusiness schema but no FAQPage. (7) Do not quote the 2021 BuildZoom rescheduling review; summarize as a pattern only if ever needed. (8) Not previously demoed or audited (repo grep clean); suppression.csv clean; GHL dedupe not run - Rozel to check before load. (9) Press release Apr 2024 came via IssueWire with a PR-vendor contact (obscured @gigs.vet) - not a company email, ignore. (10) Mixed residential + commercial/new-construction work (tenant improvements blog) - still residential-service led. (11) Open items for a second pass: Google review text + owner reply rate, LSA badge, Ad Library, owner LinkedIn, AI spot-check (D4) - any of these could move the score into SEND TODAY.</t>
+          <t>Title detail: Owner / Member (BBB Business Management) and AZ ROC Qualifying Party (BuildZoom); customers call him 'the owner Josh'; Apr-2024 press release calls him 'founder and CEO'. Legal entity note: legal: MOREHART AIR CONDITIONING AND HEATING LLC, AZ entity L14058381. (1) Route: DEMO PATH / call-first - no email exists publicly; Sam dials, asks for Josh by name; owner title on record is "Member" (BBB), he is the ROC qualifying party and works in the field. (2) Second decision-maker: Janah M Morehart, Member and registered agent (BBB details; OpenCorporates) - co-owner on record, treat as co-signer. (3) Champion/gatekeeper: Mayley Madrid, Business Development Coordinator (BBB) - praised in a site review for coordinating a same-day after-hours dispatch ("communicated with us while she worked on getting Thomas out"), so she likely owns the phone process; position the AI as after-hours/overflow only, never as replacing her. Also on record: Jeremy Robert Grubbs, Qp/Member (BuildZoom ROC-derived). Long-tenured tech Brian Sturgeon (14 yrs per a reviewer). (4) Phones: 602-640-0444 is site-only (likely RYNO tracking number, GTM present); 623-566-0005 is the number in their schema, BBB, and press - dial 623 for the office, dial 602 once after 5pm MST to hear what the tracked line actually does. Arizona has no DST (MST, UTC-7); trades window 7:00-8:30am or 4:00-5:30pm local. (5) They already collect TCPA-style SMS consent on every form, so missed-call text-back slots into an existing habit. (6) Incumbent: RYNO Strategic Solutions (HVAC-vertical web/marketing) - do not pitch web; phone + GEO wedge only; site has HVACBusiness schema but no FAQPage. (7) Do not quote the 2021 BuildZoom rescheduling review; summarize as a pattern only if ever needed. (8) Not previously demoed or audited (repo grep clean); suppression.csv clean; GHL dedupe not run - Rozel to check before load. (9) Press release Apr 2024 came via IssueWire with a PR-vendor contact (obscured @gigs.vet) - not a company email, ignore. (10) Mixed residential + commercial/new-construction work (tenant improvements blog) - still residential-service led. (11) Open items for a second pass: Google review text + owner reply rate, LSA badge, Ad Library, owner LinkedIn, AI spot-check (D4) - any of these could move the score into SEND TODAY.</t>
         </is>
       </c>
       <c r="BR22" s="10" t="inlineStr"/>
@@ -12054,7 +12054,7 @@
       </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>Owner / President ("Hey guys, this is Ricky, owner of AirBros Air Conditioning and Electrical" on the site; BBB lists "Ricardo Orta, President"; OpenCorporates registered agent "RICARDO A ORTA")</t>
+          <t>Owner / President</t>
         </is>
       </c>
       <c r="L23" s="8" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="BQ23" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: legal: AIR BROS INC; BBB: Air Bros Air Conditioning &amp; Electric. Gatekeeper/champion: Bailey McCormick, General Manager (BBB + site profile) - ask for "Ricky" (he introduces himself that way; legal name Ricardo A. Orta). Second named decision-maker on BBB: Griffin Kistler, License Holder (electrician). An unnamed brother works in the business. Legal entity AIR BROS INC, FL P20000035191, Active, registered agent Ricardo A Orta at the Delaware Ave address (OpenCorporates; Sunbiz returned 403, DBPR lookup is form-only - licenses CAC1820499 / EC13015085 not verified). No email anywhere -&gt; call-first / DEMO PATH; a written touch could go via the Facebook page or LinkedIn company page. Call the direct number 727-217-6148 (6142 is the GMB tracking line, 813-758-4044 is Podium/BBB) so the call is not credited to a paid channel. Incumbent: LeadsNearby supplies site, chat/SMS (LaunchSMS) and call tracking - never pitch a website or chat widget; voice AI is a layer, GEO only after a real audit (they track an 'OpenAI ads' source, so they are already AI-curious and may be running ChatGPT ads). Size is above the HVAC sweet spot (13 trucks, LinkedIn 11-50) - expect a numbers-first, booking-rate conversation; offer to book into their existing software. Founding year CONFLICTS (2007 / 2018 / 2020) - do not use a "since" year or anniversary opener. Community hooks: Shore Acres block parties, Stroll Snell Isle advertising partner. Best time to call: weekday mornings Eastern, before the dispatch board fills. Compliance: no cell numbers found, SMS-consent language on their forms, nothing sensitive recorded. Not checked this run (log for refresh): Google review replies, Yelp (403), Instagram (429), Facebook (login wall), Indeed/ZipRecruiter, AI spot-check, Meta Ad Library / Ads Transparency; GHL dedupe pending.</t>
+          <t>Title detail: Owner / President ("Hey guys, this is Ricky, owner of AirBros Air Conditioning and Electrical" on the site; BBB lists "Ricardo Orta, President"; OpenCorporates registered agent "RICARDO A ORTA"). Legal entity note: legal: AIR BROS INC; BBB: Air Bros Air Conditioning &amp; Electric. Gatekeeper/champion: Bailey McCormick, General Manager (BBB + site profile) - ask for "Ricky" (he introduces himself that way; legal name Ricardo A. Orta). Second named decision-maker on BBB: Griffin Kistler, License Holder (electrician). An unnamed brother works in the business. Legal entity AIR BROS INC, FL P20000035191, Active, registered agent Ricardo A Orta at the Delaware Ave address (OpenCorporates; Sunbiz returned 403, DBPR lookup is form-only - licenses CAC1820499 / EC13015085 not verified). No email anywhere -&gt; call-first / DEMO PATH; a written touch could go via the Facebook page or LinkedIn company page. Call the direct number 727-217-6148 (6142 is the GMB tracking line, 813-758-4044 is Podium/BBB) so the call is not credited to a paid channel. Incumbent: LeadsNearby supplies site, chat/SMS (LaunchSMS) and call tracking - never pitch a website or chat widget; voice AI is a layer, GEO only after a real audit (they track an 'OpenAI ads' source, so they are already AI-curious and may be running ChatGPT ads). Size is above the HVAC sweet spot (13 trucks, LinkedIn 11-50) - expect a numbers-first, booking-rate conversation; offer to book into their existing software. Founding year CONFLICTS (2007 / 2018 / 2020) - do not use a "since" year or anniversary opener. Community hooks: Shore Acres block parties, Stroll Snell Isle advertising partner. Best time to call: weekday mornings Eastern, before the dispatch board fills. Compliance: no cell numbers found, SMS-consent language on their forms, nothing sensitive recorded. Not checked this run (log for refresh): Google review replies, Yelp (403), Instagram (429), Facebook (login wall), Indeed/ZipRecruiter, AI spot-check, Meta Ad Library / Ads Transparency; GHL dedupe pending.</t>
         </is>
       </c>
       <c r="BR23" s="10" t="inlineStr"/>
@@ -12395,7 +12395,7 @@
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>Founder (About page: 'Howard Manne established The Electrician in 2004'; 'family-owned and operated'). No formal title published - 'Owner' is inferred, not stated.</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="L24" s="8" t="inlineStr">
@@ -12685,7 +12685,7 @@
       </c>
       <c r="BQ24" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: RCH Electrical, LLC. — footer reads "RCH Electric, LLC". Correction to item (1): the BBB profile for 'The Electrician' (Phillip Wills, Owner) shows 4835 Belcrest Way, Cumming GA 30040 with fax (404) 339-8500; 5490 Settingdown Rd is the GA SOS registered address for THE ELECTRICIAN, L.L.C., not the BBB address. Both still carry phone (404) 256-0169. All other notes stand.</t>
+          <t>Title detail: Founder (About page: 'Howard Manne established The Electrician in 2004'; 'family-owned and operated'). No formal title published - 'Owner' is inferred, not stated.. Legal entity note: RCH Electrical, LLC. — footer reads "RCH Electric, LLC". Correction to item (1): the BBB profile for 'The Electrician' (Phillip Wills, Owner) shows 4835 Belcrest Way, Cumming GA 30040 with fax (404) 339-8500; 5490 Settingdown Rd is the GA SOS registered address for THE ELECTRICIAN, L.L.C., not the BBB address. Both still carry phone (404) 256-0169. All other notes stand.</t>
         </is>
       </c>
       <c r="BR24" s="10" t="inlineStr"/>
@@ -12736,7 +12736,7 @@
       </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>Owner / Master Plumber (BBB: "Trent Cooke, Owner"; site About: "co-owners, Charles Wallace and Trent Cooke"; SOS via OpenCorporates: registered agent "Trent A Cooke"; 2022 press release: "owner Trent Cooke"). Co-owner: Charles Wallace (site About; LinkedIn company page).</t>
+          <t>Owner / Master Plumber</t>
         </is>
       </c>
       <c r="L25" s="8" t="inlineStr">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="BQ25" s="8" t="inlineStr">
         <is>
-          <t>Legal entity note: dba of 24/7 Plumbing Services, L.L.C.. 1) Second decision-maker: Charles Wallace, co-owner (site About; LinkedIn company page) - Sam should ask for Trent or Charles. 2) Route DEMO PATH / call-first: no email anywhere public; main line +1 281-214-9706 (site) or +1 281-391-2001 (BBB). Best window: trades 7:00-8:30 am or 4:00-5:30 pm Central. 3) Size flag: ~1,958 reviews, 7,300 sq ft warehouse, LinkedIn shows 29 associated members - likely a dispatch/office staff exists; pitch voice AI as after-hours and overflow coverage, never as replacing the office. 4) Entity: 24/7 Plumbing Services, L.L.C. (In Existence) dba 24/7 Plumbing Co., LP; the two old LP entities are merged/inactive (normal). Restated Certificate of Formation 2026-04-20 - unknown nature; do not reference in outreach. 5) Scout correction: "family-owned since 1995" belonged to Ory's Plumbing (kdhnews release) - not this company. 6) Gaps to close before SEND TODAY: GBP hours string + review text (reachability quotes, reply behavior), LSA/Google Ads check, Meta Ad Library, owner LinkedIn, and the 3x2 AI spot-check - all blocked this session by search budget/JS walls. 7) TDLR license search returned no record for RMP 37092 or "COOKE, TRENT" without the license-type selector - logged null, not a negative; RMP 37092 is self-published on the site. 8) GHL ghl-contacts.js dedupe not run here - Rozel to run before load. 9) Compliance: no cell numbers found; all numbers are business lines; "24/7 PLUMBING CO.,LP" is their registered trademark - fine to name.</t>
+          <t>Title detail: Owner / Master Plumber (BBB: "Trent Cooke, Owner"; site About: "co-owners, Charles Wallace and Trent Cooke"; SOS via OpenCorporates: registered agent "Trent A Cooke"; 2022 press release: "owner Trent Cooke"). Co-owner: Charles Wallace (site About; LinkedIn company page).. Legal entity note: dba of 24/7 Plumbing Services, L.L.C.. 1) Second decision-maker: Charles Wallace, co-owner (site About; LinkedIn company page) - Sam should ask for Trent or Charles. 2) Route DEMO PATH / call-first: no email anywhere public; main line +1 281-214-9706 (site) or +1 281-391-2001 (BBB). Best window: trades 7:00-8:30 am or 4:00-5:30 pm Central. 3) Size flag: ~1,958 reviews, 7,300 sq ft warehouse, LinkedIn shows 29 associated members - likely a dispatch/office staff exists; pitch voice AI as after-hours and overflow coverage, never as replacing the office. 4) Entity: 24/7 Plumbing Services, L.L.C. (In Existence) dba 24/7 Plumbing Co., LP; the two old LP entities are merged/inactive (normal). Restated Certificate of Formation 2026-04-20 - unknown nature; do not reference in outreach. 5) Scout correction: "family-owned since 1995" belonged to Ory's Plumbing (kdhnews release) - not this company. 6) Gaps to close before SEND TODAY: GBP hours string + review text (reachability quotes, reply behavior), LSA/Google Ads check, Meta Ad Library, owner LinkedIn, and the 3x2 AI spot-check - all blocked this session by search budget/JS walls. 7) TDLR license search returned no record for RMP 37092 or "COOKE, TRENT" without the license-type selector - logged null, not a negative; RMP 37092 is self-published on the site. 8) GHL ghl-contacts.js dedupe not run here - Rozel to run before load. 9) Compliance: no cell numbers found; all numbers are business lines; "24/7 PLUMBING CO.,LP" is their registered trademark - fine to name.</t>
         </is>
       </c>
       <c r="BR25" s="10" t="inlineStr"/>
@@ -13077,7 +13077,7 @@
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>President (BBB principal contact: 'Bill West, President' — https://www.bbb.org/us/mo/grain-valley/profile/roofing-contractors/bill-west-roofing-inc-0714-97101169); Founder/owner per site ('Founded by Bill West and now operated alongside his son Aaron' — home; 'Today Bill and his son Aaron oversee Bill West Roofing, Inc.' — /about-us/). Second decision-maker: Aaron (son; runs estimates and customer education per /about-us/; surname NOT published on any page found — do not assume).</t>
+          <t>President</t>
         </is>
       </c>
       <c r="L26" s="8" t="inlineStr">
@@ -13367,7 +13367,7 @@
       </c>
       <c r="BQ26" s="8" t="inlineStr">
         <is>
-          <t>1) Score is 54 TRUSTED = WATCH by one point; the only blocker is D4 (no AI platform could be checked). One Perplexity/ChatGPT question on 'emergency roofer near Blue Springs, MO' re-scores it to 60+ if they are not named. 2) D2 is 9, not the scout's assumed 15: the emergency page credits a human answering service — lead with 'upgrade, not replace' and the demo line, and have Sam log who actually answers after hours. 3) Owner Bill West (President per BBB) is hands-on; son Aaron runs estimates and is the likely champion — his surname is NOT published anywhere found, so address him as 'Aaron' only. 4) Only confirmed email is generic info@billwestroofing.com (in site JSON-LD, MX = Google Workspace); yahoo/gmail addresses on CertainTeed and Project Map It are third-party and need Rozel's verification before any send. 5) Google review count (~229 at 5.0) is from the Project Map It widget, not GBP — verify before quoting. 6) Founding year conflict 1976 (site) vs 1980 (BBB/Alignable) — use 'since 1976' only because it is their own claim. 7) Do not quote the site testimonial that names Brittany or any reviewer. 8) Route: call-first (Sam) because D1 = 8; the email to info@ is a secondary touch addressed to Bill and Aaron. 9) Loader must run the GHL ghl-contacts.js dedupe; not possible from this session.</t>
+          <t>Title detail: President (BBB principal contact: 'Bill West, President' — https://www.bbb.org/us/mo/grain-valley/profile/roofing-contractors/bill-west-roofing-inc-0714-97101169); Founder/owner per site ('Founded by Bill West and now operated alongside his son Aaron' — home; 'Today Bill and his son Aaron oversee Bill West Roofing, Inc.' — /about-us/). Second decision-maker: Aaron (son; runs estimates and customer education per /about-us/; surname NOT published on any page found — do not assume).. 1) Score is 54 TRUSTED = WATCH by one point; the only blocker is D4 (no AI platform could be checked). One Perplexity/ChatGPT question on 'emergency roofer near Blue Springs, MO' re-scores it to 60+ if they are not named. 2) D2 is 9, not the scout's assumed 15: the emergency page credits a human answering service — lead with 'upgrade, not replace' and the demo line, and have Sam log who actually answers after hours. 3) Owner Bill West (President per BBB) is hands-on; son Aaron runs estimates and is the likely champion — his surname is NOT published anywhere found, so address him as 'Aaron' only. 4) Only confirmed email is generic info@billwestroofing.com (in site JSON-LD, MX = Google Workspace); yahoo/gmail addresses on CertainTeed and Project Map It are third-party and need Rozel's verification before any send. 5) Google review count (~229 at 5.0) is from the Project Map It widget, not GBP — verify before quoting. 6) Founding year conflict 1976 (site) vs 1980 (BBB/Alignable) — use 'since 1976' only because it is their own claim. 7) Do not quote the site testimonial that names Brittany or any reviewer. 8) Route: call-first (Sam) because D1 = 8; the email to info@ is a secondary touch addressed to Bill and Aaron. 9) Loader must run the GHL ghl-contacts.js dedupe; not possible from this session.</t>
         </is>
       </c>
       <c r="BR26" s="10" t="inlineStr"/>

</xml_diff>

<commit_message>
Lead machine: dialable best-number extraction; CSV export and summary tools
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VEQCtkhrjvn4vtJiWBdjLw
</commit_message>
<xml_diff>
--- a/lead-machine/batches/2026-10-12-E4L-Leads-batch1.xlsx
+++ b/lead-machine/batches/2026-10-12-E4L-Leads-batch1.xlsx
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Not found (a client review says Glen shared his personal cell, but no direct line is published; main line +1 702-331-5722, fax +1 702-629-7161 per site and NV Bar)</t>
+          <t>+1 702-331-5722</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Not found (no owner cell or direct line on site, BBB, Carrier, or reviews; only the main line, fax, and the alternate 407-422-7657 office number)</t>
+          <t>+1 407-374-0779</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the main line +1 404-409-9926 is published on site, BBB and Nextdoor; line type not stated, do not text)</t>
+          <t>+1 404-409-9926</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the main line +1 770-630-6858 is published; with a 2-person crew it may be his cell — manual dial only)</t>
+          <t>+1 770-630-6858</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the main line 469-261-1503 appears on the site, BBB, JSON-LD and the TDLR record)</t>
+          <t>+1 469-261-1503</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the main line 281-907-2092 is published; the TSBPE RMP record lists no phone)</t>
+          <t>+1 281-907-2092</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>+1 405-452-0591 — LIKELY, not confirmed as owner-direct: listed as "Contact phone" under "Contact name Matt Morgan" in the May 5, 2025 GetFeatured press placement media-contact block; scout noted an older directory shows it as the Norman office line; not labeled cell/direct anywhere. Manual human dial only; line type unknown.</t>
+          <t>+1 405-452-0591</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Not found. Secondary business numbers on BBB: (704) 847-4796 (phone) and (704) 847-7301 (fax) — distinct from the site's (704) 486-2571; not tied to the owner, do not treat as a direct line.</t>
+          <t>+1 704-486-2571</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Not found (no number tied to Cynthia or Ronnie on any public page; the only numbers published are the company lines above)</t>
+          <t>+1 303-458-3790</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Not found (unlabeled second lines: +1 615-617-0513 on ProvenExpert next to the main line; +1 615-249-4851 in site service-page CTAs — neither tied to a named person)</t>
+          <t>+1 615-971-3226</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>+1 813-689-0817 (site header/contact: "call or text"; Nextdoor; Osprey Observer) — advertised as a text line, so treat as possible cell: manual human dial only, no SMS/AI voice</t>
+          <t>+1 813-689-0817</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the main line 303-759-3437 appears on site, BBB and LinkedIn)</t>
+          <t>+1 303-759-3437</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the main line +1 214-690-1941 appears on site, BBB, BuildZoom, directories; BBB lists it as "call or text")</t>
+          <t>+1 214-690-1941</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>+1 407-343-0220 (Central FL main line, 28 tel: links on site); +1 941-417-8333 (West FL / Bradenton line, footer); BBB also lists +1 877-407-2237 (toll-free, possibly legacy) and fax 866-888-9871</t>
+          <t>+1 407-343-0220</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>+1 800-356-2337 (sales, "Live Person 8am–5pm PT"); +1 707-964-5700 (local line, site footer); BBB profile lists a third number, +1 707-964-3356</t>
+          <t>+1 800-356-2337</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Not found (a second tel: link, 602-737-1788, sits behind the mobile sticky "Call" button on the site — purpose not stated; not tied to any named person, do not treat as owner-direct)</t>
+          <t>+1 602-952-8446</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Not found (NC license record phone = main line (919) 578-7798; no cell/direct line published)</t>
+          <t>+1 919-578-7798</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>+1 602-640-0444 (website header/banner/footer, tel: link x3); +1 623-566-0005 (site JSON-LD schema, BBB, Apr-2024 press release - likely the office line; the 602 number appears only on the RYNO-built site and may be a tracking number, vendor unconfirmed); +1 623-738-4004 (ServiceAgent directory mirror of Google data)</t>
+          <t>+1 602-640-0444</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Not found (only the company line and call-tracking variants are published; no cell or 'call me' line anywhere)</t>
+          <t>+1 727-217-6148</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Not found (no number is publicly tied to Trent personally; +1 713-384-3012 appears on the TDLR TABS record for the owner entity with Trent Cooke as contact, but is not labeled a direct line)</t>
+          <t>+1 281-214-9706</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Not found (neither published number is tied to Bill or Aaron by name on any page)</t>
+          <t>+1 816-295-6299</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">

</xml_diff>